<commit_message>
fixed and updated producao
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-04.xlsx
+++ b/first-atlas/producao_2026-04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFE3B84-36E0-4899-8D05-D95A00FB59FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E007CA9D-0DAC-4F89-93D0-A0D1C6A6975C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="248">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Gleicy Ferreira Gomes</t>
   </si>
   <si>
-    <t>PENDÊNCIA DOC</t>
-  </si>
-  <si>
     <t>Jamily de Lima Alves dos Santos</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>Carla Cristina de Lima Kauffmann</t>
   </si>
   <si>
-    <t>Lavinia Guimaraes Bueno</t>
-  </si>
-  <si>
     <t>Ata de eleicao da diretoria atualizada e registrado no orgao competente&lt;br&gt;&lt;br&gt;Estatuto social atualizado e registrado no orgao competente</t>
   </si>
   <si>
@@ -149,12 +143,6 @@
     <t>DS FOOD &amp; BEVARAGE LTDA</t>
   </si>
   <si>
-    <t>33708448000113</t>
-  </si>
-  <si>
-    <t>ASSOCIACAO DESPORTIVA ATHLETIC MERITI</t>
-  </si>
-  <si>
     <t>30174204000100</t>
   </si>
   <si>
@@ -200,9 +188,6 @@
     <t>CENTRO RECREATIVO ESP UNIAO AMIGOS DE VILA PROSPERIDADE</t>
   </si>
   <si>
-    <t>Procuracao da empresa . Identificamos que a representacao da sua empresa e realizada em conjunto com o tesoureiro  nomeado na clausula de administracao do contrato social e, por esse motivo, e necessario que os demais representantes tambem assinem a procuracao.&lt;br&gt;&lt;br&gt;Estatuto social atualizado e registrado no orgao competente</t>
-  </si>
-  <si>
     <t>47294711000180</t>
   </si>
   <si>
@@ -753,6 +738,51 @@
   </si>
   <si>
     <t>42.906.995 JULIANE CRISTINA DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>Ainda nao iniciou a abertura de conta</t>
+  </si>
+  <si>
+    <t>CARIMBADA</t>
+  </si>
+  <si>
+    <t>57779508000157</t>
+  </si>
+  <si>
+    <t>P V DE LIMA PEREIRA  LTDA</t>
+  </si>
+  <si>
+    <t>46974898000108</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GISELE SERAFIM </t>
+  </si>
+  <si>
+    <t>21669892000198</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NAYANA DABADIA GOMES </t>
+  </si>
+  <si>
+    <t>65984009000120</t>
+  </si>
+  <si>
+    <t>BB GESTAO E ASSESSORIA COMERCIAL LTDA</t>
+  </si>
+  <si>
+    <t>BACKOFFICE</t>
+  </si>
+  <si>
+    <t>63993426000103</t>
+  </si>
+  <si>
+    <t>MANAH ALIMENTACAO E CONSULTORIA LTDA</t>
+  </si>
+  <si>
+    <t>18669738000101</t>
+  </si>
+  <si>
+    <t>RO AMARO DECORACOES LTDA</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A45A88-3D17-4433-986A-11075963C36F}">
-  <dimension ref="A1:H99"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -1153,7 +1183,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -1170,25 +1200,25 @@
         <v>46113</v>
       </c>
       <c r="B2" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
-      </c>
-      <c r="H2" t="s">
-        <v>53</v>
+        <v>18</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -1196,22 +1226,22 @@
         <v>46113</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
         <v>7</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>233</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -1222,19 +1252,19 @@
         <v>46113</v>
       </c>
       <c r="B4" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G4" t="s">
         <v>20</v>
@@ -1248,19 +1278,19 @@
         <v>46113</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G5" t="s">
         <v>20</v>
@@ -1274,19 +1304,19 @@
         <v>46113</v>
       </c>
       <c r="B6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G6" t="s">
         <v>20</v>
@@ -1300,16 +1330,16 @@
         <v>46113</v>
       </c>
       <c r="B7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
         <v>8</v>
@@ -1326,25 +1356,25 @@
         <v>46113</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G8" t="s">
         <v>20</v>
       </c>
-      <c r="H8">
-        <v>0</v>
+      <c r="H8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -1352,25 +1382,25 @@
         <v>46113</v>
       </c>
       <c r="B9" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="D9" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G9" t="s">
         <v>20</v>
       </c>
       <c r="H9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1378,25 +1408,25 @@
         <v>46113</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="D10" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F10" t="s">
         <v>8</v>
       </c>
       <c r="G10" t="s">
-        <v>20</v>
-      </c>
-      <c r="H10" t="s">
-        <v>27</v>
+        <v>18</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -1404,16 +1434,16 @@
         <v>46113</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F11" t="s">
         <v>8</v>
@@ -1430,16 +1460,16 @@
         <v>46113</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>63</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
         <v>8</v>
@@ -1456,16 +1486,16 @@
         <v>46113</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
         <v>8</v>
@@ -1482,19 +1512,19 @@
         <v>46113</v>
       </c>
       <c r="B14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D14" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G14" t="s">
         <v>18</v>
@@ -1508,19 +1538,19 @@
         <v>46113</v>
       </c>
       <c r="B15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D15" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="E15" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>7</v>
+        <v>71</v>
       </c>
       <c r="G15" t="s">
         <v>18</v>
@@ -1534,19 +1564,19 @@
         <v>46113</v>
       </c>
       <c r="B16" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>76</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
         <v>18</v>
@@ -1560,16 +1590,16 @@
         <v>46113</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>
       </c>
       <c r="E17" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F17" t="s">
         <v>8</v>
@@ -1586,22 +1616,22 @@
         <v>46113</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C18" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D18" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F18" t="s">
         <v>8</v>
       </c>
       <c r="G18" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -1612,22 +1642,22 @@
         <v>46113</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C19" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="E19" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F19" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H19">
         <v>0</v>
@@ -1638,22 +1668,22 @@
         <v>46113</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D20" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E20" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G20" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H20">
         <v>0</v>
@@ -1664,22 +1694,22 @@
         <v>46113</v>
       </c>
       <c r="B21" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C21" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D21" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F21" t="s">
         <v>8</v>
       </c>
       <c r="G21" t="s">
-        <v>25</v>
+        <v>233</v>
       </c>
       <c r="H21">
         <v>0</v>
@@ -1690,22 +1720,22 @@
         <v>46113</v>
       </c>
       <c r="B22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C22" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F22" t="s">
         <v>8</v>
       </c>
       <c r="G22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H22">
         <v>0</v>
@@ -1716,22 +1746,22 @@
         <v>46113</v>
       </c>
       <c r="B23" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D23" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="E23" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F23" t="s">
         <v>8</v>
       </c>
       <c r="G23" t="s">
-        <v>18</v>
+        <v>233</v>
       </c>
       <c r="H23">
         <v>0</v>
@@ -1742,22 +1772,22 @@
         <v>46113</v>
       </c>
       <c r="B24" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C24" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E24" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F24" t="s">
         <v>8</v>
       </c>
       <c r="G24" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H24">
         <v>0</v>
@@ -1768,16 +1798,16 @@
         <v>46113</v>
       </c>
       <c r="B25" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E25" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F25" t="s">
         <v>8</v>
@@ -1794,16 +1824,16 @@
         <v>46113</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C26" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D26" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F26" t="s">
         <v>8</v>
@@ -1820,16 +1850,16 @@
         <v>46113</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D27" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="E27" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F27" t="s">
         <v>8</v>
@@ -1846,22 +1876,22 @@
         <v>46113</v>
       </c>
       <c r="B28" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C28" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F28" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G28" t="s">
-        <v>18</v>
+        <v>233</v>
       </c>
       <c r="H28">
         <v>0</v>
@@ -1872,22 +1902,22 @@
         <v>46113</v>
       </c>
       <c r="B29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D29" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="E29" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F29" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G29" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H29">
         <v>0</v>
@@ -1898,16 +1928,16 @@
         <v>46113</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D30" t="s">
-        <v>6</v>
+        <v>23</v>
       </c>
       <c r="E30" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F30" t="s">
         <v>8</v>
@@ -1924,22 +1954,22 @@
         <v>46113</v>
       </c>
       <c r="B31" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C31" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D31" t="s">
         <v>23</v>
       </c>
       <c r="E31" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F31" t="s">
         <v>8</v>
       </c>
       <c r="G31" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -1950,22 +1980,22 @@
         <v>46113</v>
       </c>
       <c r="B32" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D32" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="E32" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F32" t="s">
         <v>8</v>
       </c>
       <c r="G32" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -1976,19 +2006,19 @@
         <v>46113</v>
       </c>
       <c r="B33" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C33" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D33" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="E33" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F33" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G33" t="s">
         <v>18</v>
@@ -2002,19 +2032,19 @@
         <v>46113</v>
       </c>
       <c r="B34" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C34" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D34" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="E34" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F34" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G34" t="s">
         <v>18</v>
@@ -2028,16 +2058,16 @@
         <v>46113</v>
       </c>
       <c r="B35" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C35" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D35" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E35" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F35" t="s">
         <v>8</v>
@@ -2054,22 +2084,22 @@
         <v>46113</v>
       </c>
       <c r="B36" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C36" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D36" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="E36" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F36" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G36" t="s">
-        <v>18</v>
+        <v>233</v>
       </c>
       <c r="H36">
         <v>0</v>
@@ -2080,22 +2110,22 @@
         <v>46113</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C37" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D37" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="E37" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G37" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H37">
         <v>0</v>
@@ -2106,22 +2136,22 @@
         <v>46113</v>
       </c>
       <c r="B38" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C38" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D38" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E38" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F38" t="s">
         <v>8</v>
       </c>
       <c r="G38" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H38">
         <v>0</v>
@@ -2129,22 +2159,22 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B39" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C39" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D39" t="s">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="E39" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F39" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G39" t="s">
         <v>18</v>
@@ -2158,19 +2188,19 @@
         <v>46114</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C40" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D40" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="E40" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="F40" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G40" t="s">
         <v>18</v>
@@ -2184,19 +2214,19 @@
         <v>46114</v>
       </c>
       <c r="B41" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C41" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D41" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E41" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="F41" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G41" t="s">
         <v>18</v>
@@ -2210,22 +2240,25 @@
         <v>46114</v>
       </c>
       <c r="B42" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C42" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D42" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="E42" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F42" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="G42" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="H42">
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -2233,22 +2266,25 @@
         <v>46114</v>
       </c>
       <c r="B43" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C43" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D43" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E43" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F43" t="s">
         <v>8</v>
       </c>
       <c r="G43" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="H43">
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -2256,22 +2292,25 @@
         <v>46114</v>
       </c>
       <c r="B44" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C44" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D44" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="E44" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F44" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G44" t="s">
-        <v>21</v>
+        <v>18</v>
+      </c>
+      <c r="H44">
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.25">
@@ -2279,22 +2318,25 @@
         <v>46114</v>
       </c>
       <c r="B45" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C45" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D45" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="E45" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F45" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G45" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="H45">
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
@@ -2302,22 +2344,25 @@
         <v>46114</v>
       </c>
       <c r="B46" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C46" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D46" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F46" t="s">
         <v>8</v>
       </c>
       <c r="G46" t="s">
-        <v>20</v>
+        <v>18</v>
+      </c>
+      <c r="H46">
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -2325,22 +2370,25 @@
         <v>46114</v>
       </c>
       <c r="B47" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="E47" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F47" t="s">
         <v>8</v>
       </c>
       <c r="G47" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="H47">
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
@@ -2348,16 +2396,16 @@
         <v>46114</v>
       </c>
       <c r="B48" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C48" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D48" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E48" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="F48" t="s">
         <v>8</v>
@@ -2365,1178 +2413,1443 @@
       <c r="G48" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>46114</v>
       </c>
       <c r="B49" t="s">
+        <v>138</v>
+      </c>
+      <c r="C49" t="s">
+        <v>139</v>
+      </c>
+      <c r="D49" t="s">
+        <v>31</v>
+      </c>
+      <c r="E49" t="s">
+        <v>39</v>
+      </c>
+      <c r="F49" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" t="s">
+        <v>233</v>
+      </c>
+      <c r="H49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B50" t="s">
+        <v>140</v>
+      </c>
+      <c r="C50" t="s">
         <v>141</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D50" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" t="s">
+        <v>37</v>
+      </c>
+      <c r="F50" t="s">
+        <v>8</v>
+      </c>
+      <c r="G50" t="s">
+        <v>21</v>
+      </c>
+      <c r="H50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B51" t="s">
         <v>142</v>
       </c>
-      <c r="D49" t="s">
-        <v>15</v>
-      </c>
-      <c r="E49" t="s">
+      <c r="C51" t="s">
+        <v>143</v>
+      </c>
+      <c r="D51" t="s">
+        <v>14</v>
+      </c>
+      <c r="E51" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51" t="s">
+        <v>8</v>
+      </c>
+      <c r="G51" t="s">
+        <v>18</v>
+      </c>
+      <c r="H51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B52" t="s">
+        <v>34</v>
+      </c>
+      <c r="C52" t="s">
+        <v>35</v>
+      </c>
+      <c r="D52" t="s">
+        <v>9</v>
+      </c>
+      <c r="E52" t="s">
+        <v>39</v>
+      </c>
+      <c r="F52" t="s">
+        <v>7</v>
+      </c>
+      <c r="G52" t="s">
+        <v>233</v>
+      </c>
+      <c r="H52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B53" t="s">
+        <v>144</v>
+      </c>
+      <c r="C53" t="s">
+        <v>145</v>
+      </c>
+      <c r="D53" t="s">
+        <v>16</v>
+      </c>
+      <c r="E53" t="s">
+        <v>37</v>
+      </c>
+      <c r="F53" t="s">
+        <v>8</v>
+      </c>
+      <c r="G53" t="s">
+        <v>18</v>
+      </c>
+      <c r="H53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B54" t="s">
+        <v>146</v>
+      </c>
+      <c r="C54" t="s">
+        <v>147</v>
+      </c>
+      <c r="D54" t="s">
+        <v>14</v>
+      </c>
+      <c r="E54" t="s">
+        <v>37</v>
+      </c>
+      <c r="F54" t="s">
+        <v>8</v>
+      </c>
+      <c r="G54" t="s">
+        <v>18</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B55" t="s">
+        <v>148</v>
+      </c>
+      <c r="C55" t="s">
+        <v>149</v>
+      </c>
+      <c r="D55" t="s">
         <v>41</v>
       </c>
-      <c r="F49" t="s">
-        <v>8</v>
-      </c>
-      <c r="G49" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B50" t="s">
-        <v>143</v>
-      </c>
-      <c r="C50" t="s">
-        <v>144</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="E55" t="s">
+        <v>39</v>
+      </c>
+      <c r="F55" t="s">
+        <v>7</v>
+      </c>
+      <c r="G55" t="s">
+        <v>18</v>
+      </c>
+      <c r="H55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B56" t="s">
+        <v>150</v>
+      </c>
+      <c r="C56" t="s">
+        <v>151</v>
+      </c>
+      <c r="D56" t="s">
+        <v>31</v>
+      </c>
+      <c r="E56" t="s">
+        <v>39</v>
+      </c>
+      <c r="F56" t="s">
+        <v>8</v>
+      </c>
+      <c r="G56" t="s">
+        <v>18</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B57" t="s">
+        <v>152</v>
+      </c>
+      <c r="C57" t="s">
+        <v>153</v>
+      </c>
+      <c r="D57" t="s">
+        <v>40</v>
+      </c>
+      <c r="E57" t="s">
+        <v>39</v>
+      </c>
+      <c r="F57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" t="s">
+        <v>18</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B58" t="s">
+        <v>42</v>
+      </c>
+      <c r="C58" t="s">
+        <v>154</v>
+      </c>
+      <c r="D58" t="s">
+        <v>22</v>
+      </c>
+      <c r="E58" t="s">
+        <v>39</v>
+      </c>
+      <c r="F58" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" t="s">
+        <v>18</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B59" t="s">
+        <v>155</v>
+      </c>
+      <c r="C59" t="s">
+        <v>156</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" t="s">
+        <v>37</v>
+      </c>
+      <c r="F59" t="s">
+        <v>8</v>
+      </c>
+      <c r="G59" t="s">
+        <v>18</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B60" t="s">
+        <v>157</v>
+      </c>
+      <c r="C60" t="s">
+        <v>158</v>
+      </c>
+      <c r="D60" t="s">
+        <v>14</v>
+      </c>
+      <c r="E60" t="s">
+        <v>37</v>
+      </c>
+      <c r="F60" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" t="s">
+        <v>18</v>
+      </c>
+      <c r="H60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B61" t="s">
+        <v>159</v>
+      </c>
+      <c r="C61" t="s">
+        <v>160</v>
+      </c>
+      <c r="D61" t="s">
+        <v>23</v>
+      </c>
+      <c r="E61" t="s">
+        <v>37</v>
+      </c>
+      <c r="F61" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" t="s">
+        <v>18</v>
+      </c>
+      <c r="H61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B62" t="s">
+        <v>32</v>
+      </c>
+      <c r="C62" t="s">
         <v>33</v>
-      </c>
-      <c r="E50" t="s">
-        <v>43</v>
-      </c>
-      <c r="F50" t="s">
-        <v>8</v>
-      </c>
-      <c r="G50" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B51" t="s">
-        <v>145</v>
-      </c>
-      <c r="C51" t="s">
-        <v>146</v>
-      </c>
-      <c r="D51" t="s">
-        <v>15</v>
-      </c>
-      <c r="E51" t="s">
-        <v>41</v>
-      </c>
-      <c r="F51" t="s">
-        <v>8</v>
-      </c>
-      <c r="G51" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B52" t="s">
-        <v>147</v>
-      </c>
-      <c r="C52" t="s">
-        <v>148</v>
-      </c>
-      <c r="D52" t="s">
-        <v>14</v>
-      </c>
-      <c r="E52" t="s">
-        <v>41</v>
-      </c>
-      <c r="F52" t="s">
-        <v>8</v>
-      </c>
-      <c r="G52" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B53" t="s">
-        <v>38</v>
-      </c>
-      <c r="C53" t="s">
-        <v>39</v>
-      </c>
-      <c r="D53" t="s">
-        <v>9</v>
-      </c>
-      <c r="E53" t="s">
-        <v>43</v>
-      </c>
-      <c r="F53" t="s">
-        <v>7</v>
-      </c>
-      <c r="G53" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B54" t="s">
-        <v>149</v>
-      </c>
-      <c r="C54" t="s">
-        <v>150</v>
-      </c>
-      <c r="D54" t="s">
-        <v>16</v>
-      </c>
-      <c r="E54" t="s">
-        <v>41</v>
-      </c>
-      <c r="F54" t="s">
-        <v>8</v>
-      </c>
-      <c r="G54" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B55" t="s">
-        <v>151</v>
-      </c>
-      <c r="C55" t="s">
-        <v>152</v>
-      </c>
-      <c r="D55" t="s">
-        <v>14</v>
-      </c>
-      <c r="E55" t="s">
-        <v>41</v>
-      </c>
-      <c r="F55" t="s">
-        <v>8</v>
-      </c>
-      <c r="G55" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B56" t="s">
-        <v>153</v>
-      </c>
-      <c r="C56" t="s">
-        <v>154</v>
-      </c>
-      <c r="D56" t="s">
-        <v>45</v>
-      </c>
-      <c r="E56" t="s">
-        <v>43</v>
-      </c>
-      <c r="F56" t="s">
-        <v>7</v>
-      </c>
-      <c r="G56" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B57" t="s">
-        <v>155</v>
-      </c>
-      <c r="C57" t="s">
-        <v>156</v>
-      </c>
-      <c r="D57" t="s">
-        <v>33</v>
-      </c>
-      <c r="E57" t="s">
-        <v>43</v>
-      </c>
-      <c r="F57" t="s">
-        <v>8</v>
-      </c>
-      <c r="G57" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B58" t="s">
-        <v>157</v>
-      </c>
-      <c r="C58" t="s">
-        <v>158</v>
-      </c>
-      <c r="D58" t="s">
-        <v>44</v>
-      </c>
-      <c r="E58" t="s">
-        <v>43</v>
-      </c>
-      <c r="F58" t="s">
-        <v>7</v>
-      </c>
-      <c r="G58" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B59" t="s">
-        <v>46</v>
-      </c>
-      <c r="C59" t="s">
-        <v>159</v>
-      </c>
-      <c r="D59" t="s">
-        <v>22</v>
-      </c>
-      <c r="E59" t="s">
-        <v>43</v>
-      </c>
-      <c r="F59" t="s">
-        <v>8</v>
-      </c>
-      <c r="G59" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B60" t="s">
-        <v>160</v>
-      </c>
-      <c r="C60" t="s">
-        <v>161</v>
-      </c>
-      <c r="D60" t="s">
-        <v>11</v>
-      </c>
-      <c r="E60" t="s">
-        <v>41</v>
-      </c>
-      <c r="F60" t="s">
-        <v>8</v>
-      </c>
-      <c r="G60" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B61" t="s">
-        <v>162</v>
-      </c>
-      <c r="C61" t="s">
-        <v>163</v>
-      </c>
-      <c r="D61" t="s">
-        <v>14</v>
-      </c>
-      <c r="E61" t="s">
-        <v>41</v>
-      </c>
-      <c r="F61" t="s">
-        <v>8</v>
-      </c>
-      <c r="G61" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B62" t="s">
-        <v>164</v>
-      </c>
-      <c r="C62" t="s">
-        <v>165</v>
       </c>
       <c r="D62" t="s">
         <v>23</v>
       </c>
       <c r="E62" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="F62" t="s">
         <v>8</v>
       </c>
       <c r="G62" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="H62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
         <v>46114</v>
       </c>
       <c r="B63" t="s">
-        <v>34</v>
+        <v>161</v>
       </c>
       <c r="C63" t="s">
-        <v>35</v>
+        <v>162</v>
       </c>
       <c r="D63" t="s">
+        <v>40</v>
+      </c>
+      <c r="E63" t="s">
+        <v>39</v>
+      </c>
+      <c r="F63" t="s">
+        <v>7</v>
+      </c>
+      <c r="G63" t="s">
+        <v>233</v>
+      </c>
+      <c r="H63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B64" t="s">
+        <v>163</v>
+      </c>
+      <c r="C64" t="s">
+        <v>164</v>
+      </c>
+      <c r="D64" t="s">
         <v>23</v>
       </c>
-      <c r="E63" t="s">
-        <v>41</v>
-      </c>
-      <c r="F63" t="s">
-        <v>8</v>
-      </c>
-      <c r="G63" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B64" t="s">
+      <c r="E64" t="s">
+        <v>37</v>
+      </c>
+      <c r="F64" t="s">
+        <v>8</v>
+      </c>
+      <c r="G64" t="s">
+        <v>18</v>
+      </c>
+      <c r="H64">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B65" t="s">
+        <v>165</v>
+      </c>
+      <c r="C65" t="s">
         <v>166</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D65" t="s">
+        <v>16</v>
+      </c>
+      <c r="E65" t="s">
+        <v>37</v>
+      </c>
+      <c r="F65" t="s">
+        <v>8</v>
+      </c>
+      <c r="G65" t="s">
+        <v>18</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B66" t="s">
         <v>167</v>
       </c>
-      <c r="D64" t="s">
-        <v>44</v>
-      </c>
-      <c r="E64" t="s">
-        <v>43</v>
-      </c>
-      <c r="F64" t="s">
-        <v>7</v>
-      </c>
-      <c r="G64" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A65" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B65" t="s">
+      <c r="C66" t="s">
         <v>168</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D66" t="s">
+        <v>6</v>
+      </c>
+      <c r="E66" t="s">
+        <v>37</v>
+      </c>
+      <c r="F66" t="s">
+        <v>8</v>
+      </c>
+      <c r="G66" t="s">
+        <v>18</v>
+      </c>
+      <c r="H66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B67" t="s">
         <v>169</v>
       </c>
-      <c r="D65" t="s">
-        <v>23</v>
-      </c>
-      <c r="E65" t="s">
-        <v>41</v>
-      </c>
-      <c r="F65" t="s">
-        <v>8</v>
-      </c>
-      <c r="G65" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B66" t="s">
+      <c r="C67" t="s">
         <v>170</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D67" t="s">
+        <v>22</v>
+      </c>
+      <c r="E67" t="s">
+        <v>39</v>
+      </c>
+      <c r="F67" t="s">
+        <v>8</v>
+      </c>
+      <c r="G67" t="s">
+        <v>18</v>
+      </c>
+      <c r="H67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B68" t="s">
         <v>171</v>
       </c>
-      <c r="D66" t="s">
-        <v>16</v>
-      </c>
-      <c r="E66" t="s">
-        <v>41</v>
-      </c>
-      <c r="F66" t="s">
-        <v>8</v>
-      </c>
-      <c r="G66" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B67" t="s">
+      <c r="C68" t="s">
         <v>172</v>
-      </c>
-      <c r="C67" t="s">
-        <v>173</v>
-      </c>
-      <c r="D67" t="s">
-        <v>6</v>
-      </c>
-      <c r="E67" t="s">
-        <v>41</v>
-      </c>
-      <c r="F67" t="s">
-        <v>8</v>
-      </c>
-      <c r="G67" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B68" t="s">
-        <v>174</v>
-      </c>
-      <c r="C68" t="s">
-        <v>175</v>
       </c>
       <c r="D68" t="s">
         <v>22</v>
       </c>
       <c r="E68" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F68" t="s">
         <v>8</v>
       </c>
       <c r="G68" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="H68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
         <v>46114</v>
       </c>
       <c r="B69" t="s">
+        <v>173</v>
+      </c>
+      <c r="C69" t="s">
+        <v>174</v>
+      </c>
+      <c r="D69" t="s">
+        <v>40</v>
+      </c>
+      <c r="E69" t="s">
+        <v>39</v>
+      </c>
+      <c r="F69" t="s">
+        <v>7</v>
+      </c>
+      <c r="G69" t="s">
+        <v>18</v>
+      </c>
+      <c r="H69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B70" t="s">
+        <v>175</v>
+      </c>
+      <c r="C70" t="s">
         <v>176</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D70" t="s">
+        <v>31</v>
+      </c>
+      <c r="E70" t="s">
+        <v>39</v>
+      </c>
+      <c r="F70" t="s">
+        <v>8</v>
+      </c>
+      <c r="G70" t="s">
+        <v>21</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B71" t="s">
         <v>177</v>
       </c>
-      <c r="D69" t="s">
-        <v>22</v>
-      </c>
-      <c r="E69" t="s">
-        <v>43</v>
-      </c>
-      <c r="F69" t="s">
-        <v>8</v>
-      </c>
-      <c r="G69" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B70" t="s">
+      <c r="C71" t="s">
         <v>178</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D71" t="s">
+        <v>14</v>
+      </c>
+      <c r="E71" t="s">
+        <v>37</v>
+      </c>
+      <c r="F71" t="s">
+        <v>8</v>
+      </c>
+      <c r="G71" t="s">
+        <v>18</v>
+      </c>
+      <c r="H71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B72" t="s">
         <v>179</v>
       </c>
-      <c r="D70" t="s">
-        <v>44</v>
-      </c>
-      <c r="E70" t="s">
-        <v>43</v>
-      </c>
-      <c r="F70" t="s">
+      <c r="C72" t="s">
+        <v>180</v>
+      </c>
+      <c r="D72" t="s">
+        <v>40</v>
+      </c>
+      <c r="E72" t="s">
+        <v>39</v>
+      </c>
+      <c r="F72" t="s">
         <v>7</v>
-      </c>
-      <c r="G70" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B71" t="s">
-        <v>180</v>
-      </c>
-      <c r="C71" t="s">
-        <v>181</v>
-      </c>
-      <c r="D71" t="s">
-        <v>33</v>
-      </c>
-      <c r="E71" t="s">
-        <v>43</v>
-      </c>
-      <c r="F71" t="s">
-        <v>8</v>
-      </c>
-      <c r="G71" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A72" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B72" t="s">
-        <v>182</v>
-      </c>
-      <c r="C72" t="s">
-        <v>183</v>
-      </c>
-      <c r="D72" t="s">
-        <v>14</v>
-      </c>
-      <c r="E72" t="s">
-        <v>41</v>
-      </c>
-      <c r="F72" t="s">
-        <v>8</v>
       </c>
       <c r="G72" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H72" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
         <v>46114</v>
       </c>
       <c r="B73" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C73" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D73" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E73" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F73" t="s">
         <v>7</v>
       </c>
       <c r="G73" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="H73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>46114</v>
       </c>
       <c r="B74" t="s">
+        <v>183</v>
+      </c>
+      <c r="C74" t="s">
+        <v>184</v>
+      </c>
+      <c r="D74" t="s">
+        <v>31</v>
+      </c>
+      <c r="E74" t="s">
+        <v>39</v>
+      </c>
+      <c r="F74" t="s">
+        <v>8</v>
+      </c>
+      <c r="G74" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B75" t="s">
+        <v>185</v>
+      </c>
+      <c r="C75" t="s">
         <v>186</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D75" t="s">
+        <v>14</v>
+      </c>
+      <c r="E75" t="s">
+        <v>37</v>
+      </c>
+      <c r="F75" t="s">
+        <v>8</v>
+      </c>
+      <c r="G75" t="s">
+        <v>18</v>
+      </c>
+      <c r="H75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B76" t="s">
         <v>187</v>
       </c>
-      <c r="D74" t="s">
-        <v>45</v>
-      </c>
-      <c r="E74" t="s">
-        <v>43</v>
-      </c>
-      <c r="F74" t="s">
+      <c r="C76" t="s">
+        <v>188</v>
+      </c>
+      <c r="D76" t="s">
+        <v>15</v>
+      </c>
+      <c r="E76" t="s">
+        <v>37</v>
+      </c>
+      <c r="F76" t="s">
+        <v>8</v>
+      </c>
+      <c r="G76" t="s">
+        <v>18</v>
+      </c>
+      <c r="H76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B77" t="s">
+        <v>189</v>
+      </c>
+      <c r="C77" t="s">
+        <v>190</v>
+      </c>
+      <c r="D77" t="s">
+        <v>11</v>
+      </c>
+      <c r="E77" t="s">
+        <v>37</v>
+      </c>
+      <c r="F77" t="s">
+        <v>8</v>
+      </c>
+      <c r="G77" t="s">
+        <v>18</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B78" t="s">
+        <v>191</v>
+      </c>
+      <c r="C78" t="s">
+        <v>192</v>
+      </c>
+      <c r="D78" t="s">
+        <v>14</v>
+      </c>
+      <c r="E78" t="s">
+        <v>37</v>
+      </c>
+      <c r="F78" t="s">
+        <v>8</v>
+      </c>
+      <c r="G78" t="s">
+        <v>18</v>
+      </c>
+      <c r="H78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B79" t="s">
+        <v>193</v>
+      </c>
+      <c r="C79" t="s">
+        <v>194</v>
+      </c>
+      <c r="D79" t="s">
+        <v>11</v>
+      </c>
+      <c r="E79" t="s">
+        <v>37</v>
+      </c>
+      <c r="F79" t="s">
+        <v>8</v>
+      </c>
+      <c r="G79" t="s">
+        <v>18</v>
+      </c>
+      <c r="H79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B80" t="s">
+        <v>195</v>
+      </c>
+      <c r="C80" t="s">
+        <v>196</v>
+      </c>
+      <c r="D80" t="s">
+        <v>6</v>
+      </c>
+      <c r="E80" t="s">
+        <v>37</v>
+      </c>
+      <c r="F80" t="s">
+        <v>8</v>
+      </c>
+      <c r="G80" t="s">
+        <v>18</v>
+      </c>
+      <c r="H80">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B81" t="s">
+        <v>197</v>
+      </c>
+      <c r="C81" t="s">
+        <v>198</v>
+      </c>
+      <c r="D81" t="s">
+        <v>9</v>
+      </c>
+      <c r="E81" t="s">
+        <v>39</v>
+      </c>
+      <c r="F81" t="s">
         <v>7</v>
       </c>
-      <c r="G74" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B75" t="s">
-        <v>188</v>
-      </c>
-      <c r="C75" t="s">
-        <v>189</v>
-      </c>
-      <c r="D75" t="s">
-        <v>33</v>
-      </c>
-      <c r="E75" t="s">
-        <v>43</v>
-      </c>
-      <c r="F75" t="s">
-        <v>8</v>
-      </c>
-      <c r="G75" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B76" t="s">
-        <v>190</v>
-      </c>
-      <c r="C76" t="s">
-        <v>191</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="G81" t="s">
+        <v>233</v>
+      </c>
+      <c r="H81">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B82" t="s">
+        <v>199</v>
+      </c>
+      <c r="C82" t="s">
+        <v>200</v>
+      </c>
+      <c r="D82" t="s">
+        <v>28</v>
+      </c>
+      <c r="E82" t="s">
+        <v>37</v>
+      </c>
+      <c r="F82" t="s">
+        <v>8</v>
+      </c>
+      <c r="G82" t="s">
+        <v>18</v>
+      </c>
+      <c r="H82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B83" t="s">
+        <v>201</v>
+      </c>
+      <c r="C83" t="s">
+        <v>202</v>
+      </c>
+      <c r="D83" t="s">
+        <v>15</v>
+      </c>
+      <c r="E83" t="s">
+        <v>37</v>
+      </c>
+      <c r="F83" t="s">
+        <v>8</v>
+      </c>
+      <c r="G83" t="s">
+        <v>18</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B84" t="s">
+        <v>203</v>
+      </c>
+      <c r="C84" t="s">
+        <v>204</v>
+      </c>
+      <c r="D84" t="s">
         <v>14</v>
       </c>
-      <c r="E76" t="s">
-        <v>41</v>
-      </c>
-      <c r="F76" t="s">
-        <v>8</v>
-      </c>
-      <c r="G76" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B77" t="s">
-        <v>192</v>
-      </c>
-      <c r="C77" t="s">
-        <v>193</v>
-      </c>
-      <c r="D77" t="s">
+      <c r="E84" t="s">
+        <v>37</v>
+      </c>
+      <c r="F84" t="s">
+        <v>8</v>
+      </c>
+      <c r="G84" t="s">
+        <v>18</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B85" t="s">
+        <v>205</v>
+      </c>
+      <c r="C85" t="s">
+        <v>206</v>
+      </c>
+      <c r="D85" t="s">
+        <v>19</v>
+      </c>
+      <c r="E85" t="s">
+        <v>37</v>
+      </c>
+      <c r="F85" t="s">
+        <v>8</v>
+      </c>
+      <c r="G85" t="s">
+        <v>18</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B86" t="s">
+        <v>207</v>
+      </c>
+      <c r="C86" t="s">
+        <v>208</v>
+      </c>
+      <c r="D86" t="s">
+        <v>28</v>
+      </c>
+      <c r="E86" t="s">
+        <v>37</v>
+      </c>
+      <c r="F86" t="s">
+        <v>8</v>
+      </c>
+      <c r="G86" t="s">
+        <v>18</v>
+      </c>
+      <c r="H86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B87" t="s">
+        <v>209</v>
+      </c>
+      <c r="C87" t="s">
+        <v>210</v>
+      </c>
+      <c r="D87" t="s">
         <v>15</v>
       </c>
-      <c r="E77" t="s">
-        <v>41</v>
-      </c>
-      <c r="F77" t="s">
-        <v>8</v>
-      </c>
-      <c r="G77" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B78" t="s">
-        <v>194</v>
-      </c>
-      <c r="C78" t="s">
-        <v>195</v>
-      </c>
-      <c r="D78" t="s">
+      <c r="E87" t="s">
+        <v>37</v>
+      </c>
+      <c r="F87" t="s">
+        <v>8</v>
+      </c>
+      <c r="G87" t="s">
+        <v>233</v>
+      </c>
+      <c r="H87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B88" t="s">
+        <v>211</v>
+      </c>
+      <c r="C88" t="s">
+        <v>212</v>
+      </c>
+      <c r="D88" t="s">
         <v>11</v>
       </c>
-      <c r="E78" t="s">
-        <v>41</v>
-      </c>
-      <c r="F78" t="s">
-        <v>8</v>
-      </c>
-      <c r="G78" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B79" t="s">
-        <v>196</v>
-      </c>
-      <c r="C79" t="s">
-        <v>197</v>
-      </c>
-      <c r="D79" t="s">
+      <c r="E88" t="s">
+        <v>37</v>
+      </c>
+      <c r="F88" t="s">
+        <v>8</v>
+      </c>
+      <c r="G88" t="s">
+        <v>18</v>
+      </c>
+      <c r="H88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B89" t="s">
+        <v>213</v>
+      </c>
+      <c r="C89" t="s">
+        <v>214</v>
+      </c>
+      <c r="D89" t="s">
+        <v>16</v>
+      </c>
+      <c r="E89" t="s">
+        <v>37</v>
+      </c>
+      <c r="F89" t="s">
+        <v>8</v>
+      </c>
+      <c r="G89" t="s">
+        <v>233</v>
+      </c>
+      <c r="H89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B90" t="s">
+        <v>215</v>
+      </c>
+      <c r="C90" t="s">
+        <v>216</v>
+      </c>
+      <c r="D90" t="s">
+        <v>24</v>
+      </c>
+      <c r="E90" t="s">
+        <v>39</v>
+      </c>
+      <c r="F90" t="s">
+        <v>7</v>
+      </c>
+      <c r="G90" t="s">
+        <v>18</v>
+      </c>
+      <c r="H90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B91" t="s">
+        <v>217</v>
+      </c>
+      <c r="C91" t="s">
+        <v>218</v>
+      </c>
+      <c r="D91" t="s">
+        <v>22</v>
+      </c>
+      <c r="E91" t="s">
+        <v>39</v>
+      </c>
+      <c r="F91" t="s">
+        <v>8</v>
+      </c>
+      <c r="G91" t="s">
+        <v>21</v>
+      </c>
+      <c r="H91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B92" t="s">
+        <v>219</v>
+      </c>
+      <c r="C92" t="s">
+        <v>220</v>
+      </c>
+      <c r="D92" t="s">
         <v>14</v>
       </c>
-      <c r="E79" t="s">
-        <v>41</v>
-      </c>
-      <c r="F79" t="s">
-        <v>8</v>
-      </c>
-      <c r="G79" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A80" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B80" t="s">
-        <v>198</v>
-      </c>
-      <c r="C80" t="s">
-        <v>199</v>
-      </c>
-      <c r="D80" t="s">
-        <v>11</v>
-      </c>
-      <c r="E80" t="s">
-        <v>41</v>
-      </c>
-      <c r="F80" t="s">
-        <v>8</v>
-      </c>
-      <c r="G80" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A81" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B81" t="s">
-        <v>200</v>
-      </c>
-      <c r="C81" t="s">
-        <v>201</v>
-      </c>
-      <c r="D81" t="s">
+      <c r="E92" t="s">
+        <v>37</v>
+      </c>
+      <c r="F92" t="s">
+        <v>8</v>
+      </c>
+      <c r="G92" t="s">
+        <v>18</v>
+      </c>
+      <c r="H92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B93" t="s">
+        <v>221</v>
+      </c>
+      <c r="C93" t="s">
+        <v>222</v>
+      </c>
+      <c r="D93" t="s">
+        <v>25</v>
+      </c>
+      <c r="E93" t="s">
+        <v>39</v>
+      </c>
+      <c r="F93" t="s">
+        <v>10</v>
+      </c>
+      <c r="G93" t="s">
+        <v>18</v>
+      </c>
+      <c r="H93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B94" t="s">
+        <v>223</v>
+      </c>
+      <c r="C94" t="s">
+        <v>224</v>
+      </c>
+      <c r="D94" t="s">
+        <v>14</v>
+      </c>
+      <c r="E94" t="s">
+        <v>37</v>
+      </c>
+      <c r="F94" t="s">
+        <v>8</v>
+      </c>
+      <c r="G94" t="s">
+        <v>18</v>
+      </c>
+      <c r="H94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B95" t="s">
+        <v>225</v>
+      </c>
+      <c r="C95" t="s">
+        <v>226</v>
+      </c>
+      <c r="D95" t="s">
+        <v>16</v>
+      </c>
+      <c r="E95" t="s">
+        <v>37</v>
+      </c>
+      <c r="F95" t="s">
+        <v>8</v>
+      </c>
+      <c r="G95" t="s">
+        <v>18</v>
+      </c>
+      <c r="H95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B96" t="s">
+        <v>227</v>
+      </c>
+      <c r="C96" t="s">
+        <v>228</v>
+      </c>
+      <c r="D96" t="s">
+        <v>19</v>
+      </c>
+      <c r="E96" t="s">
+        <v>37</v>
+      </c>
+      <c r="F96" t="s">
+        <v>8</v>
+      </c>
+      <c r="G96" t="s">
+        <v>18</v>
+      </c>
+      <c r="H96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B97" t="s">
+        <v>229</v>
+      </c>
+      <c r="C97" t="s">
+        <v>230</v>
+      </c>
+      <c r="D97" t="s">
+        <v>25</v>
+      </c>
+      <c r="E97" t="s">
+        <v>39</v>
+      </c>
+      <c r="F97" t="s">
+        <v>8</v>
+      </c>
+      <c r="G97" t="s">
+        <v>18</v>
+      </c>
+      <c r="H97">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>46114</v>
+      </c>
+      <c r="B98" t="s">
+        <v>231</v>
+      </c>
+      <c r="C98" t="s">
+        <v>232</v>
+      </c>
+      <c r="D98" t="s">
+        <v>16</v>
+      </c>
+      <c r="E98" t="s">
+        <v>37</v>
+      </c>
+      <c r="F98" t="s">
+        <v>8</v>
+      </c>
+      <c r="G98" t="s">
+        <v>18</v>
+      </c>
+      <c r="H98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B99" t="s">
+        <v>235</v>
+      </c>
+      <c r="C99" t="s">
+        <v>236</v>
+      </c>
+      <c r="D99" t="s">
+        <v>24</v>
+      </c>
+      <c r="F99" t="s">
+        <v>7</v>
+      </c>
+      <c r="G99" t="s">
+        <v>18</v>
+      </c>
+      <c r="H99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B100" t="s">
+        <v>237</v>
+      </c>
+      <c r="C100" t="s">
+        <v>238</v>
+      </c>
+      <c r="D100" t="s">
+        <v>19</v>
+      </c>
+      <c r="F100" t="s">
+        <v>8</v>
+      </c>
+      <c r="G100" t="s">
+        <v>18</v>
+      </c>
+      <c r="H100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B101" t="s">
+        <v>239</v>
+      </c>
+      <c r="C101" t="s">
+        <v>240</v>
+      </c>
+      <c r="D101" t="s">
         <v>6</v>
       </c>
-      <c r="E81" t="s">
-        <v>41</v>
-      </c>
-      <c r="F81" t="s">
-        <v>8</v>
-      </c>
-      <c r="G81" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B82" t="s">
-        <v>202</v>
-      </c>
-      <c r="C82" t="s">
-        <v>203</v>
-      </c>
-      <c r="D82" t="s">
-        <v>9</v>
-      </c>
-      <c r="E82" t="s">
-        <v>43</v>
-      </c>
-      <c r="F82" t="s">
-        <v>7</v>
-      </c>
-      <c r="G82" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A83" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B83" t="s">
-        <v>204</v>
-      </c>
-      <c r="C83" t="s">
-        <v>205</v>
-      </c>
-      <c r="D83" t="s">
-        <v>29</v>
-      </c>
-      <c r="E83" t="s">
-        <v>41</v>
-      </c>
-      <c r="F83" t="s">
-        <v>8</v>
-      </c>
-      <c r="G83" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A84" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B84" t="s">
-        <v>206</v>
-      </c>
-      <c r="C84" t="s">
-        <v>207</v>
-      </c>
-      <c r="D84" t="s">
-        <v>15</v>
-      </c>
-      <c r="E84" t="s">
-        <v>41</v>
-      </c>
-      <c r="F84" t="s">
-        <v>8</v>
-      </c>
-      <c r="G84" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A85" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B85" t="s">
-        <v>208</v>
-      </c>
-      <c r="C85" t="s">
-        <v>209</v>
-      </c>
-      <c r="D85" t="s">
-        <v>14</v>
-      </c>
-      <c r="E85" t="s">
-        <v>41</v>
-      </c>
-      <c r="F85" t="s">
-        <v>8</v>
-      </c>
-      <c r="G85" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B86" t="s">
-        <v>210</v>
-      </c>
-      <c r="C86" t="s">
-        <v>211</v>
-      </c>
-      <c r="D86" t="s">
-        <v>19</v>
-      </c>
-      <c r="E86" t="s">
-        <v>41</v>
-      </c>
-      <c r="F86" t="s">
-        <v>8</v>
-      </c>
-      <c r="G86" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A87" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B87" t="s">
-        <v>212</v>
-      </c>
-      <c r="C87" t="s">
-        <v>213</v>
-      </c>
-      <c r="D87" t="s">
-        <v>29</v>
-      </c>
-      <c r="E87" t="s">
-        <v>41</v>
-      </c>
-      <c r="F87" t="s">
-        <v>8</v>
-      </c>
-      <c r="G87" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B88" t="s">
-        <v>214</v>
-      </c>
-      <c r="C88" t="s">
-        <v>215</v>
-      </c>
-      <c r="D88" t="s">
-        <v>15</v>
-      </c>
-      <c r="E88" t="s">
-        <v>41</v>
-      </c>
-      <c r="F88" t="s">
-        <v>8</v>
-      </c>
-      <c r="G88" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B89" t="s">
-        <v>216</v>
-      </c>
-      <c r="C89" t="s">
-        <v>217</v>
-      </c>
-      <c r="D89" t="s">
-        <v>11</v>
-      </c>
-      <c r="E89" t="s">
-        <v>41</v>
-      </c>
-      <c r="F89" t="s">
-        <v>8</v>
-      </c>
-      <c r="G89" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A90" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B90" t="s">
-        <v>218</v>
-      </c>
-      <c r="C90" t="s">
-        <v>219</v>
-      </c>
-      <c r="D90" t="s">
-        <v>16</v>
-      </c>
-      <c r="E90" t="s">
-        <v>41</v>
-      </c>
-      <c r="F90" t="s">
-        <v>8</v>
-      </c>
-      <c r="G90" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A91" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B91" t="s">
-        <v>220</v>
-      </c>
-      <c r="C91" t="s">
-        <v>221</v>
-      </c>
-      <c r="D91" t="s">
-        <v>24</v>
-      </c>
-      <c r="E91" t="s">
-        <v>43</v>
-      </c>
-      <c r="F91" t="s">
-        <v>7</v>
-      </c>
-      <c r="G91" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A92" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B92" t="s">
-        <v>222</v>
-      </c>
-      <c r="C92" t="s">
-        <v>223</v>
-      </c>
-      <c r="D92" t="s">
-        <v>22</v>
-      </c>
-      <c r="E92" t="s">
-        <v>43</v>
-      </c>
-      <c r="F92" t="s">
-        <v>8</v>
-      </c>
-      <c r="G92" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A93" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B93" t="s">
-        <v>224</v>
-      </c>
-      <c r="C93" t="s">
-        <v>225</v>
-      </c>
-      <c r="D93" t="s">
-        <v>14</v>
-      </c>
-      <c r="E93" t="s">
-        <v>41</v>
-      </c>
-      <c r="F93" t="s">
-        <v>8</v>
-      </c>
-      <c r="G93" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A94" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B94" t="s">
-        <v>226</v>
-      </c>
-      <c r="C94" t="s">
-        <v>227</v>
-      </c>
-      <c r="D94" t="s">
-        <v>26</v>
-      </c>
-      <c r="E94" t="s">
-        <v>43</v>
-      </c>
-      <c r="F94" t="s">
-        <v>10</v>
-      </c>
-      <c r="G94" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A95" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B95" t="s">
-        <v>228</v>
-      </c>
-      <c r="C95" t="s">
-        <v>229</v>
-      </c>
-      <c r="D95" t="s">
-        <v>14</v>
-      </c>
-      <c r="E95" t="s">
-        <v>41</v>
-      </c>
-      <c r="F95" t="s">
-        <v>8</v>
-      </c>
-      <c r="G95" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A96" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B96" t="s">
-        <v>230</v>
-      </c>
-      <c r="C96" t="s">
-        <v>231</v>
-      </c>
-      <c r="D96" t="s">
-        <v>16</v>
-      </c>
-      <c r="E96" t="s">
-        <v>41</v>
-      </c>
-      <c r="F96" t="s">
-        <v>8</v>
-      </c>
-      <c r="G96" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A97" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B97" t="s">
-        <v>232</v>
-      </c>
-      <c r="C97" t="s">
-        <v>233</v>
-      </c>
-      <c r="D97" t="s">
-        <v>19</v>
-      </c>
-      <c r="E97" t="s">
-        <v>41</v>
-      </c>
-      <c r="F97" t="s">
-        <v>8</v>
-      </c>
-      <c r="G97" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A98" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B98" t="s">
-        <v>234</v>
-      </c>
-      <c r="C98" t="s">
-        <v>235</v>
-      </c>
-      <c r="D98" t="s">
-        <v>26</v>
-      </c>
-      <c r="E98" t="s">
-        <v>43</v>
-      </c>
-      <c r="F98" t="s">
-        <v>8</v>
-      </c>
-      <c r="G98" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A99" s="1">
-        <v>46114</v>
-      </c>
-      <c r="B99" t="s">
-        <v>236</v>
-      </c>
-      <c r="C99" t="s">
-        <v>237</v>
-      </c>
-      <c r="D99" t="s">
-        <v>16</v>
-      </c>
-      <c r="E99" t="s">
-        <v>41</v>
-      </c>
-      <c r="F99" t="s">
-        <v>8</v>
-      </c>
-      <c r="G99" t="s">
-        <v>20</v>
+      <c r="F101" t="s">
+        <v>8</v>
+      </c>
+      <c r="G101" t="s">
+        <v>18</v>
+      </c>
+      <c r="H101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B102" t="s">
+        <v>241</v>
+      </c>
+      <c r="C102" t="s">
+        <v>242</v>
+      </c>
+      <c r="D102" t="s">
+        <v>27</v>
+      </c>
+      <c r="F102" t="s">
+        <v>243</v>
+      </c>
+      <c r="G102" t="s">
+        <v>18</v>
+      </c>
+      <c r="H102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B103" t="s">
+        <v>244</v>
+      </c>
+      <c r="C103" t="s">
+        <v>245</v>
+      </c>
+      <c r="D103" t="s">
+        <v>27</v>
+      </c>
+      <c r="F103" t="s">
+        <v>8</v>
+      </c>
+      <c r="G103" t="s">
+        <v>18</v>
+      </c>
+      <c r="H103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B104" t="s">
+        <v>246</v>
+      </c>
+      <c r="C104" t="s">
+        <v>247</v>
+      </c>
+      <c r="D104" t="s">
+        <v>6</v>
+      </c>
+      <c r="F104" t="s">
+        <v>8</v>
+      </c>
+      <c r="G104" t="s">
+        <v>18</v>
+      </c>
+      <c r="H104">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated balde and producao - base 06/04/2026
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-04.xlsx
+++ b/first-atlas/producao_2026-04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E007CA9D-0DAC-4F89-93D0-A0D1C6A6975C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47B3935-63A7-43F2-A66A-0FAFDECA49C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1109" uniqueCount="411">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -783,6 +783,495 @@
   </si>
   <si>
     <t>RO AMARO DECORACOES LTDA</t>
+  </si>
+  <si>
+    <t>35448429000120</t>
+  </si>
+  <si>
+    <t>A P DE OLIVEIRA DRINKS</t>
+  </si>
+  <si>
+    <t>61243990000183</t>
+  </si>
+  <si>
+    <t>23805136000174</t>
+  </si>
+  <si>
+    <t>47021542000104</t>
+  </si>
+  <si>
+    <t>47.021.542 MARCELO SEBASTIAO DA SILVA</t>
+  </si>
+  <si>
+    <t>VISAO ATACADO 2025 LTDA</t>
+  </si>
+  <si>
+    <t>53169061000143</t>
+  </si>
+  <si>
+    <t>HAMILTON FERREIRA SANTOS</t>
+  </si>
+  <si>
+    <t>62911781000123</t>
+  </si>
+  <si>
+    <t>LUCAS ALEXANDRE DA SILVA</t>
+  </si>
+  <si>
+    <t>45813756000198</t>
+  </si>
+  <si>
+    <t>GISLAINE DOS SANTOS OLIVEIRA ENXOVAIS</t>
+  </si>
+  <si>
+    <t>36692888000118</t>
+  </si>
+  <si>
+    <t>DALVA TOLOTO DA SILVA</t>
+  </si>
+  <si>
+    <t>52836638000160</t>
+  </si>
+  <si>
+    <t>JONATHAN LIMA COSTA</t>
+  </si>
+  <si>
+    <t>60393286000144</t>
+  </si>
+  <si>
+    <t>ELIVELTON LINHARES CAMPOS</t>
+  </si>
+  <si>
+    <t>Sophia Bagagi Pigente</t>
+  </si>
+  <si>
+    <t>43353024000137</t>
+  </si>
+  <si>
+    <t>DUDU MED LTDA</t>
+  </si>
+  <si>
+    <t>42124483000186</t>
+  </si>
+  <si>
+    <t>DANIEL SOSO DOS SANTOS</t>
+  </si>
+  <si>
+    <t>62380827000125</t>
+  </si>
+  <si>
+    <t>JOAO AUGUSTO GUSMIN</t>
+  </si>
+  <si>
+    <t>Mensageria</t>
+  </si>
+  <si>
+    <t>63516613000104</t>
+  </si>
+  <si>
+    <t>MIGUEL DE OLIVEIRA HELIODORO</t>
+  </si>
+  <si>
+    <t>42278873000100</t>
+  </si>
+  <si>
+    <t>PEMASA ACIONAMENTOS EM VENDAS LTDA</t>
+  </si>
+  <si>
+    <t>38209501000155</t>
+  </si>
+  <si>
+    <t>RAYLENA ANGELI FERREIRA SOUSA LTDA</t>
+  </si>
+  <si>
+    <t>45673721000109</t>
+  </si>
+  <si>
+    <t>JANAINA PETRY DIAS ARAUJO</t>
+  </si>
+  <si>
+    <t>44855510000116</t>
+  </si>
+  <si>
+    <t>FABRICIO DA SILVA BORGES</t>
+  </si>
+  <si>
+    <t>42082269000104</t>
+  </si>
+  <si>
+    <t>CARDOSO REFORMAS E CONSTRUCOES LTDA</t>
+  </si>
+  <si>
+    <t>35627147000190</t>
+  </si>
+  <si>
+    <t>KAIO DIAS BRAGA</t>
+  </si>
+  <si>
+    <t>62918441000124</t>
+  </si>
+  <si>
+    <t>DELLICATO MOVEIS RUSTICOS LTDA</t>
+  </si>
+  <si>
+    <t>21792653000120</t>
+  </si>
+  <si>
+    <t>AGNALDO LOPES DE OLIVEIRA JUNIOR</t>
+  </si>
+  <si>
+    <t>29691416000185</t>
+  </si>
+  <si>
+    <t>VILMA C DOS SANTOS</t>
+  </si>
+  <si>
+    <t>60662949000189</t>
+  </si>
+  <si>
+    <t>FABRICIO RODRIGUES FERREIRA LTDA</t>
+  </si>
+  <si>
+    <t>24904741000165</t>
+  </si>
+  <si>
+    <t>FABIO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>44174304000140</t>
+  </si>
+  <si>
+    <t>L. W. INTERMEDIACOES E PARANA REPASSES DE VEICULOS LTDA</t>
+  </si>
+  <si>
+    <t>35348212000149</t>
+  </si>
+  <si>
+    <t>BARBEARIA ROBSON RODRIGUES LTDA</t>
+  </si>
+  <si>
+    <t>40729151000108</t>
+  </si>
+  <si>
+    <t>VERA MARIA ALVES</t>
+  </si>
+  <si>
+    <t>51918690000101</t>
+  </si>
+  <si>
+    <t>GD ADMINISTRACAO DE IMOVEIS LTDA</t>
+  </si>
+  <si>
+    <t>63196651000119</t>
+  </si>
+  <si>
+    <t>ERICK VINICIUS PEREIRA</t>
+  </si>
+  <si>
+    <t>48972361000126</t>
+  </si>
+  <si>
+    <t>48.972.361 MARCOS JUNIOR LEMOS QUADROS</t>
+  </si>
+  <si>
+    <t>MARCO AURELIO FERNANDESQUADROS</t>
+  </si>
+  <si>
+    <t>53945967000102</t>
+  </si>
+  <si>
+    <t>53.945.967 JOHN WARLLEY PERES DA CUNHA</t>
+  </si>
+  <si>
+    <t>35909090000112</t>
+  </si>
+  <si>
+    <t>TOME P PEIXOTO CONSULTORIA E ASSESSORIA EM GESTAO PUBLICA E PRIVADA</t>
+  </si>
+  <si>
+    <t>26055903000163</t>
+  </si>
+  <si>
+    <t>CLAUDIA KELLY DE PAULA CARONI</t>
+  </si>
+  <si>
+    <t>40795819000107</t>
+  </si>
+  <si>
+    <t>40.795.819 JOAO VITOR FERREIRA</t>
+  </si>
+  <si>
+    <t>64736462000154</t>
+  </si>
+  <si>
+    <t>HUB SERV LTDA</t>
+  </si>
+  <si>
+    <t>43080997000140</t>
+  </si>
+  <si>
+    <t>GEORGE ALBERTO SILVA</t>
+  </si>
+  <si>
+    <t>58450219000172</t>
+  </si>
+  <si>
+    <t>FILIPE SOUZA WISNIEWSKI</t>
+  </si>
+  <si>
+    <t>54700991000144</t>
+  </si>
+  <si>
+    <t>L H R M TEIXEIRA REPRESENTACOES</t>
+  </si>
+  <si>
+    <t>25316150000130</t>
+  </si>
+  <si>
+    <t>MANOEL TRANSPORTE E TURISMO LTDA</t>
+  </si>
+  <si>
+    <t>34594623000151</t>
+  </si>
+  <si>
+    <t>34.594.623 MARIA TAIS ALVES FERREIRA</t>
+  </si>
+  <si>
+    <t>55487148000194</t>
+  </si>
+  <si>
+    <t>BRAVENICA CLINIC LTDA</t>
+  </si>
+  <si>
+    <t>43424148000166</t>
+  </si>
+  <si>
+    <t>GALO PINTURAS LTDA</t>
+  </si>
+  <si>
+    <t>33775001000167</t>
+  </si>
+  <si>
+    <t>ALUIZIO DA FRANCA SAMPAIO NETO LTDA</t>
+  </si>
+  <si>
+    <t>35480368000189</t>
+  </si>
+  <si>
+    <t>35.480.368 JOSE MARCIO DE OLIVEIRA FELIPE</t>
+  </si>
+  <si>
+    <t>58746440000172</t>
+  </si>
+  <si>
+    <t>58.746.440 FERNANDA MOURA DA COSTA</t>
+  </si>
+  <si>
+    <t>62829235000148</t>
+  </si>
+  <si>
+    <t>RENOVE TEXTURA E GRAFIATOS LTDA</t>
+  </si>
+  <si>
+    <t>43350059000112</t>
+  </si>
+  <si>
+    <t>M SALES DA COSTA</t>
+  </si>
+  <si>
+    <t>60398871000137</t>
+  </si>
+  <si>
+    <t>FREE-LANCER APOIO E CONSULTORIA EM LOGISTICA LTDA</t>
+  </si>
+  <si>
+    <t>26365461000151</t>
+  </si>
+  <si>
+    <t>AA ESTILO LTDA</t>
+  </si>
+  <si>
+    <t>33936185000108</t>
+  </si>
+  <si>
+    <t>DANILO ENIO FERREIRA RODRIGUES</t>
+  </si>
+  <si>
+    <t>15640609000100</t>
+  </si>
+  <si>
+    <t>15.640.609 DIOGO JOSE PIRES FERREIRA E SILVA</t>
+  </si>
+  <si>
+    <t>58612131000100</t>
+  </si>
+  <si>
+    <t>58.612.131 EVANDRO SANTOS NUNES</t>
+  </si>
+  <si>
+    <t>46351752000106</t>
+  </si>
+  <si>
+    <t>MARILANE V. DA SILVA TRANSPORTES</t>
+  </si>
+  <si>
+    <t>62931198000184</t>
+  </si>
+  <si>
+    <t>62.931.198 PYETTRO PEREIRA SANTOS</t>
+  </si>
+  <si>
+    <t>57379665000175</t>
+  </si>
+  <si>
+    <t>RONALDO DE SOUSA BARBOSA</t>
+  </si>
+  <si>
+    <t>07587995000188</t>
+  </si>
+  <si>
+    <t>ELIO PEREIRA NEVES</t>
+  </si>
+  <si>
+    <t>42636556000119</t>
+  </si>
+  <si>
+    <t>42.636.556 ADRIANA FELIZARDO DA SILVA ANDRADE</t>
+  </si>
+  <si>
+    <t>53275325000143</t>
+  </si>
+  <si>
+    <t>ADRIANA BARBOSA DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>54644628000159</t>
+  </si>
+  <si>
+    <t>VALDIR FERREIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>41408783000124</t>
+  </si>
+  <si>
+    <t>JOSE MARIEL GOIS DA SILVA</t>
+  </si>
+  <si>
+    <t>21808221000160</t>
+  </si>
+  <si>
+    <t>JACKSON DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>48436958000156</t>
+  </si>
+  <si>
+    <t>DOUGLAS P. DA SILVA MANUTENCAO E REPARACAO LTDA</t>
+  </si>
+  <si>
+    <t>04950823000139</t>
+  </si>
+  <si>
+    <t>LUCIANO GUERRA</t>
+  </si>
+  <si>
+    <t>29680418000179</t>
+  </si>
+  <si>
+    <t>FLAVIO MAIA DOS REIS</t>
+  </si>
+  <si>
+    <t>59397317000156</t>
+  </si>
+  <si>
+    <t>59.397.317 CIRENIO ALVES DE SOUSA</t>
+  </si>
+  <si>
+    <t>23791623000125</t>
+  </si>
+  <si>
+    <t>ROJAKE GUSTAVO GUIMARAES DA SILVA</t>
+  </si>
+  <si>
+    <t>24596809000196</t>
+  </si>
+  <si>
+    <t>24.596.809 GRAZIELLE FERNANDA RIBEIRO</t>
+  </si>
+  <si>
+    <t>27299033000130</t>
+  </si>
+  <si>
+    <t>RAFAELA LISANDRA DE OLIVEIRA FREITAS</t>
+  </si>
+  <si>
+    <t>46802938000126</t>
+  </si>
+  <si>
+    <t>SAVIO BARBOSA SANTOS</t>
+  </si>
+  <si>
+    <t>66094998000149</t>
+  </si>
+  <si>
+    <t>JULIA MAIA LIPPI SOCIEDADE INDIVIDUAL DE ADVOCACIA</t>
+  </si>
+  <si>
+    <t>LEAD MANUAL</t>
+  </si>
+  <si>
+    <t>23551126000150</t>
+  </si>
+  <si>
+    <t>JULIANA ARAUJO SALES PILATES</t>
+  </si>
+  <si>
+    <t>47814690000186</t>
+  </si>
+  <si>
+    <t>CARLOS IZUILO MEIRELES GOMES</t>
+  </si>
+  <si>
+    <t>41861083000190</t>
+  </si>
+  <si>
+    <t>MARCELO SANTOS SILVA</t>
+  </si>
+  <si>
+    <t>58382829000186</t>
+  </si>
+  <si>
+    <t>GOLDEN COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>43802995000117</t>
+  </si>
+  <si>
+    <t>CEREALISTA ARVORE DA VIDA MEDICINA NATURAL LTDA</t>
+  </si>
+  <si>
+    <t>28075940000169</t>
+  </si>
+  <si>
+    <t>PAULO CESAR MACHADO</t>
+  </si>
+  <si>
+    <t>52542837000166</t>
+  </si>
+  <si>
+    <t>THAYNA CRISTHYNA DA SILVA MORAIS</t>
+  </si>
+  <si>
+    <t>40385373000142</t>
+  </si>
+  <si>
+    <t>GABRIEL HENRIQUE DE SOUSA</t>
+  </si>
+  <si>
+    <t>58325459000145</t>
+  </si>
+  <si>
+    <t>58.325.459 GENAILDO DE SOUZA SANTOS</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A45A88-3D17-4433-986A-11075963C36F}">
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H184"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -3727,6 +4216,9 @@
       <c r="D99" t="s">
         <v>24</v>
       </c>
+      <c r="E99" t="s">
+        <v>39</v>
+      </c>
       <c r="F99" t="s">
         <v>7</v>
       </c>
@@ -3750,6 +4242,9 @@
       <c r="D100" t="s">
         <v>19</v>
       </c>
+      <c r="E100" t="s">
+        <v>37</v>
+      </c>
       <c r="F100" t="s">
         <v>8</v>
       </c>
@@ -3773,6 +4268,9 @@
       <c r="D101" t="s">
         <v>6</v>
       </c>
+      <c r="E101" t="s">
+        <v>37</v>
+      </c>
       <c r="F101" t="s">
         <v>8</v>
       </c>
@@ -3796,6 +4294,9 @@
       <c r="D102" t="s">
         <v>27</v>
       </c>
+      <c r="E102" t="s">
+        <v>38</v>
+      </c>
       <c r="F102" t="s">
         <v>243</v>
       </c>
@@ -3819,6 +4320,9 @@
       <c r="D103" t="s">
         <v>27</v>
       </c>
+      <c r="E103" t="s">
+        <v>38</v>
+      </c>
       <c r="F103" t="s">
         <v>8</v>
       </c>
@@ -3842,6 +4346,9 @@
       <c r="D104" t="s">
         <v>6</v>
       </c>
+      <c r="E104" t="s">
+        <v>37</v>
+      </c>
       <c r="F104" t="s">
         <v>8</v>
       </c>
@@ -3850,6 +4357,1846 @@
       </c>
       <c r="H104">
         <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B105" t="s">
+        <v>252</v>
+      </c>
+      <c r="C105" t="s">
+        <v>253</v>
+      </c>
+      <c r="D105" t="s">
+        <v>28</v>
+      </c>
+      <c r="E105" t="s">
+        <v>37</v>
+      </c>
+      <c r="F105" t="s">
+        <v>8</v>
+      </c>
+      <c r="G105" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B106" t="s">
+        <v>248</v>
+      </c>
+      <c r="C106" t="s">
+        <v>249</v>
+      </c>
+      <c r="D106" t="s">
+        <v>31</v>
+      </c>
+      <c r="E106" t="s">
+        <v>39</v>
+      </c>
+      <c r="F106" t="s">
+        <v>8</v>
+      </c>
+      <c r="G106" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B107" t="s">
+        <v>250</v>
+      </c>
+      <c r="C107" t="s">
+        <v>254</v>
+      </c>
+      <c r="D107" t="s">
+        <v>31</v>
+      </c>
+      <c r="E107" t="s">
+        <v>39</v>
+      </c>
+      <c r="F107" t="s">
+        <v>8</v>
+      </c>
+      <c r="G107" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B108" t="s">
+        <v>255</v>
+      </c>
+      <c r="C108" t="s">
+        <v>256</v>
+      </c>
+      <c r="D108" t="s">
+        <v>14</v>
+      </c>
+      <c r="E108" t="s">
+        <v>37</v>
+      </c>
+      <c r="F108" t="s">
+        <v>8</v>
+      </c>
+      <c r="G108" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B109" t="s">
+        <v>257</v>
+      </c>
+      <c r="C109" t="s">
+        <v>258</v>
+      </c>
+      <c r="D109" t="s">
+        <v>6</v>
+      </c>
+      <c r="E109" t="s">
+        <v>37</v>
+      </c>
+      <c r="F109" t="s">
+        <v>8</v>
+      </c>
+      <c r="G109" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B110" t="s">
+        <v>259</v>
+      </c>
+      <c r="C110" t="s">
+        <v>260</v>
+      </c>
+      <c r="D110" t="s">
+        <v>15</v>
+      </c>
+      <c r="E110" t="s">
+        <v>37</v>
+      </c>
+      <c r="F110" t="s">
+        <v>8</v>
+      </c>
+      <c r="G110" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B111" t="s">
+        <v>261</v>
+      </c>
+      <c r="C111" t="s">
+        <v>262</v>
+      </c>
+      <c r="D111" t="s">
+        <v>16</v>
+      </c>
+      <c r="E111" t="s">
+        <v>37</v>
+      </c>
+      <c r="F111" t="s">
+        <v>8</v>
+      </c>
+      <c r="G111" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B112" t="s">
+        <v>263</v>
+      </c>
+      <c r="C112" t="s">
+        <v>264</v>
+      </c>
+      <c r="D112" t="s">
+        <v>12</v>
+      </c>
+      <c r="E112" t="s">
+        <v>37</v>
+      </c>
+      <c r="F112" t="s">
+        <v>8</v>
+      </c>
+      <c r="G112" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B113" t="s">
+        <v>265</v>
+      </c>
+      <c r="C113" t="s">
+        <v>266</v>
+      </c>
+      <c r="D113" t="s">
+        <v>267</v>
+      </c>
+      <c r="E113" t="s">
+        <v>37</v>
+      </c>
+      <c r="F113" t="s">
+        <v>7</v>
+      </c>
+      <c r="G113" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B114" t="s">
+        <v>268</v>
+      </c>
+      <c r="C114" t="s">
+        <v>269</v>
+      </c>
+      <c r="D114" t="s">
+        <v>9</v>
+      </c>
+      <c r="E114" t="s">
+        <v>39</v>
+      </c>
+      <c r="F114" t="s">
+        <v>7</v>
+      </c>
+      <c r="G114" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B115" t="s">
+        <v>270</v>
+      </c>
+      <c r="C115" t="s">
+        <v>271</v>
+      </c>
+      <c r="D115" t="s">
+        <v>6</v>
+      </c>
+      <c r="E115" t="s">
+        <v>37</v>
+      </c>
+      <c r="F115" t="s">
+        <v>8</v>
+      </c>
+      <c r="G115" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B116" t="s">
+        <v>272</v>
+      </c>
+      <c r="C116" t="s">
+        <v>273</v>
+      </c>
+      <c r="D116" t="s">
+        <v>14</v>
+      </c>
+      <c r="E116" t="s">
+        <v>37</v>
+      </c>
+      <c r="F116" t="s">
+        <v>274</v>
+      </c>
+      <c r="G116" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B117" t="s">
+        <v>275</v>
+      </c>
+      <c r="C117" t="s">
+        <v>276</v>
+      </c>
+      <c r="D117" t="s">
+        <v>23</v>
+      </c>
+      <c r="E117" t="s">
+        <v>37</v>
+      </c>
+      <c r="F117" t="s">
+        <v>8</v>
+      </c>
+      <c r="G117" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B118" t="s">
+        <v>277</v>
+      </c>
+      <c r="C118" t="s">
+        <v>278</v>
+      </c>
+      <c r="D118" t="s">
+        <v>6</v>
+      </c>
+      <c r="E118" t="s">
+        <v>37</v>
+      </c>
+      <c r="F118" t="s">
+        <v>8</v>
+      </c>
+      <c r="G118" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A119" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B119" t="s">
+        <v>279</v>
+      </c>
+      <c r="C119" t="s">
+        <v>280</v>
+      </c>
+      <c r="D119" t="s">
+        <v>267</v>
+      </c>
+      <c r="E119" t="s">
+        <v>37</v>
+      </c>
+      <c r="F119" t="s">
+        <v>8</v>
+      </c>
+      <c r="G119" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A120" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B120" t="s">
+        <v>281</v>
+      </c>
+      <c r="C120" t="s">
+        <v>282</v>
+      </c>
+      <c r="D120" t="s">
+        <v>24</v>
+      </c>
+      <c r="E120" t="s">
+        <v>39</v>
+      </c>
+      <c r="F120" t="s">
+        <v>7</v>
+      </c>
+      <c r="G120" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A121" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B121" t="s">
+        <v>283</v>
+      </c>
+      <c r="C121" t="s">
+        <v>284</v>
+      </c>
+      <c r="D121" t="s">
+        <v>267</v>
+      </c>
+      <c r="E121" t="s">
+        <v>37</v>
+      </c>
+      <c r="F121" t="s">
+        <v>8</v>
+      </c>
+      <c r="G121" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A122" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B122" t="s">
+        <v>285</v>
+      </c>
+      <c r="C122" t="s">
+        <v>286</v>
+      </c>
+      <c r="D122" t="s">
+        <v>15</v>
+      </c>
+      <c r="E122" t="s">
+        <v>37</v>
+      </c>
+      <c r="F122" t="s">
+        <v>8</v>
+      </c>
+      <c r="G122" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A123" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B123" t="s">
+        <v>287</v>
+      </c>
+      <c r="C123" t="s">
+        <v>288</v>
+      </c>
+      <c r="D123" t="s">
+        <v>16</v>
+      </c>
+      <c r="E123" t="s">
+        <v>37</v>
+      </c>
+      <c r="F123" t="s">
+        <v>8</v>
+      </c>
+      <c r="G123" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A124" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B124" t="s">
+        <v>289</v>
+      </c>
+      <c r="C124" t="s">
+        <v>290</v>
+      </c>
+      <c r="D124" t="s">
+        <v>11</v>
+      </c>
+      <c r="E124" t="s">
+        <v>37</v>
+      </c>
+      <c r="F124" t="s">
+        <v>8</v>
+      </c>
+      <c r="G124" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A125" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B125" t="s">
+        <v>291</v>
+      </c>
+      <c r="C125" t="s">
+        <v>292</v>
+      </c>
+      <c r="D125" t="s">
+        <v>28</v>
+      </c>
+      <c r="E125" t="s">
+        <v>37</v>
+      </c>
+      <c r="F125" t="s">
+        <v>8</v>
+      </c>
+      <c r="G125" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A126" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B126" t="s">
+        <v>293</v>
+      </c>
+      <c r="C126" t="s">
+        <v>294</v>
+      </c>
+      <c r="D126" t="s">
+        <v>23</v>
+      </c>
+      <c r="E126" t="s">
+        <v>37</v>
+      </c>
+      <c r="F126" t="s">
+        <v>8</v>
+      </c>
+      <c r="G126" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A127" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B127" t="s">
+        <v>295</v>
+      </c>
+      <c r="C127" t="s">
+        <v>296</v>
+      </c>
+      <c r="D127" t="s">
+        <v>14</v>
+      </c>
+      <c r="E127" t="s">
+        <v>37</v>
+      </c>
+      <c r="F127" t="s">
+        <v>8</v>
+      </c>
+      <c r="G127" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A128" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B128" t="s">
+        <v>297</v>
+      </c>
+      <c r="C128" t="s">
+        <v>298</v>
+      </c>
+      <c r="D128" t="s">
+        <v>28</v>
+      </c>
+      <c r="E128" t="s">
+        <v>37</v>
+      </c>
+      <c r="F128" t="s">
+        <v>8</v>
+      </c>
+      <c r="G128" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A129" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B129" t="s">
+        <v>299</v>
+      </c>
+      <c r="C129" t="s">
+        <v>300</v>
+      </c>
+      <c r="D129" t="s">
+        <v>16</v>
+      </c>
+      <c r="E129" t="s">
+        <v>37</v>
+      </c>
+      <c r="F129" t="s">
+        <v>8</v>
+      </c>
+      <c r="G129" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A130" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B130" t="s">
+        <v>301</v>
+      </c>
+      <c r="C130" t="s">
+        <v>302</v>
+      </c>
+      <c r="D130" t="s">
+        <v>22</v>
+      </c>
+      <c r="E130" t="s">
+        <v>39</v>
+      </c>
+      <c r="F130" t="s">
+        <v>7</v>
+      </c>
+      <c r="G130" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A131" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B131" t="s">
+        <v>303</v>
+      </c>
+      <c r="C131" t="s">
+        <v>304</v>
+      </c>
+      <c r="D131" t="s">
+        <v>24</v>
+      </c>
+      <c r="E131" t="s">
+        <v>39</v>
+      </c>
+      <c r="F131" t="s">
+        <v>7</v>
+      </c>
+      <c r="G131" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A132" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B132" t="s">
+        <v>305</v>
+      </c>
+      <c r="C132" t="s">
+        <v>306</v>
+      </c>
+      <c r="D132" t="s">
+        <v>11</v>
+      </c>
+      <c r="E132" t="s">
+        <v>37</v>
+      </c>
+      <c r="F132" t="s">
+        <v>8</v>
+      </c>
+      <c r="G132" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A133" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B133" t="s">
+        <v>307</v>
+      </c>
+      <c r="C133" t="s">
+        <v>308</v>
+      </c>
+      <c r="D133" t="s">
+        <v>24</v>
+      </c>
+      <c r="E133" t="s">
+        <v>39</v>
+      </c>
+      <c r="F133" t="s">
+        <v>7</v>
+      </c>
+      <c r="G133" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A134" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B134" t="s">
+        <v>309</v>
+      </c>
+      <c r="C134" t="s">
+        <v>310</v>
+      </c>
+      <c r="D134" t="s">
+        <v>16</v>
+      </c>
+      <c r="E134" t="s">
+        <v>37</v>
+      </c>
+      <c r="F134" t="s">
+        <v>8</v>
+      </c>
+      <c r="G134" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A135" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B135" t="s">
+        <v>251</v>
+      </c>
+      <c r="C135" t="s">
+        <v>311</v>
+      </c>
+      <c r="D135" t="s">
+        <v>9</v>
+      </c>
+      <c r="E135" t="s">
+        <v>39</v>
+      </c>
+      <c r="F135" t="s">
+        <v>8</v>
+      </c>
+      <c r="G135" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A136" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B136" t="s">
+        <v>312</v>
+      </c>
+      <c r="C136" t="s">
+        <v>313</v>
+      </c>
+      <c r="D136" t="s">
+        <v>28</v>
+      </c>
+      <c r="E136" t="s">
+        <v>37</v>
+      </c>
+      <c r="F136" t="s">
+        <v>8</v>
+      </c>
+      <c r="G136" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A137" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B137" t="s">
+        <v>314</v>
+      </c>
+      <c r="C137" t="s">
+        <v>315</v>
+      </c>
+      <c r="D137" t="s">
+        <v>23</v>
+      </c>
+      <c r="E137" t="s">
+        <v>37</v>
+      </c>
+      <c r="F137" t="s">
+        <v>8</v>
+      </c>
+      <c r="G137" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A138" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B138" t="s">
+        <v>316</v>
+      </c>
+      <c r="C138" t="s">
+        <v>317</v>
+      </c>
+      <c r="D138" t="s">
+        <v>12</v>
+      </c>
+      <c r="E138" t="s">
+        <v>37</v>
+      </c>
+      <c r="F138" t="s">
+        <v>8</v>
+      </c>
+      <c r="G138" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A139" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B139" t="s">
+        <v>318</v>
+      </c>
+      <c r="C139" t="s">
+        <v>319</v>
+      </c>
+      <c r="D139" t="s">
+        <v>16</v>
+      </c>
+      <c r="E139" t="s">
+        <v>37</v>
+      </c>
+      <c r="F139" t="s">
+        <v>8</v>
+      </c>
+      <c r="G139" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A140" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B140" t="s">
+        <v>320</v>
+      </c>
+      <c r="C140" t="s">
+        <v>321</v>
+      </c>
+      <c r="D140" t="s">
+        <v>11</v>
+      </c>
+      <c r="E140" t="s">
+        <v>37</v>
+      </c>
+      <c r="F140" t="s">
+        <v>8</v>
+      </c>
+      <c r="G140" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A141" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B141" t="s">
+        <v>322</v>
+      </c>
+      <c r="C141" t="s">
+        <v>323</v>
+      </c>
+      <c r="D141" t="s">
+        <v>6</v>
+      </c>
+      <c r="E141" t="s">
+        <v>37</v>
+      </c>
+      <c r="F141" t="s">
+        <v>8</v>
+      </c>
+      <c r="G141" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A142" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B142" t="s">
+        <v>324</v>
+      </c>
+      <c r="C142" t="s">
+        <v>325</v>
+      </c>
+      <c r="D142" t="s">
+        <v>12</v>
+      </c>
+      <c r="E142" t="s">
+        <v>37</v>
+      </c>
+      <c r="F142" t="s">
+        <v>8</v>
+      </c>
+      <c r="G142" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A143" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B143" t="s">
+        <v>326</v>
+      </c>
+      <c r="C143" t="s">
+        <v>327</v>
+      </c>
+      <c r="D143" t="s">
+        <v>9</v>
+      </c>
+      <c r="E143" t="s">
+        <v>39</v>
+      </c>
+      <c r="F143" t="s">
+        <v>7</v>
+      </c>
+      <c r="G143" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A144" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B144" t="s">
+        <v>328</v>
+      </c>
+      <c r="C144" t="s">
+        <v>329</v>
+      </c>
+      <c r="D144" t="s">
+        <v>31</v>
+      </c>
+      <c r="E144" t="s">
+        <v>39</v>
+      </c>
+      <c r="F144" t="s">
+        <v>8</v>
+      </c>
+      <c r="G144" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A145" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B145" t="s">
+        <v>330</v>
+      </c>
+      <c r="C145" t="s">
+        <v>331</v>
+      </c>
+      <c r="D145" t="s">
+        <v>14</v>
+      </c>
+      <c r="E145" t="s">
+        <v>37</v>
+      </c>
+      <c r="F145" t="s">
+        <v>8</v>
+      </c>
+      <c r="G145" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A146" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B146" t="s">
+        <v>332</v>
+      </c>
+      <c r="C146" t="s">
+        <v>333</v>
+      </c>
+      <c r="D146" t="s">
+        <v>15</v>
+      </c>
+      <c r="E146" t="s">
+        <v>37</v>
+      </c>
+      <c r="F146" t="s">
+        <v>8</v>
+      </c>
+      <c r="G146" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A147" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B147" t="s">
+        <v>334</v>
+      </c>
+      <c r="C147" t="s">
+        <v>335</v>
+      </c>
+      <c r="D147" t="s">
+        <v>31</v>
+      </c>
+      <c r="E147" t="s">
+        <v>39</v>
+      </c>
+      <c r="F147" t="s">
+        <v>8</v>
+      </c>
+      <c r="G147" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B148" t="s">
+        <v>336</v>
+      </c>
+      <c r="C148" t="s">
+        <v>337</v>
+      </c>
+      <c r="D148" t="s">
+        <v>14</v>
+      </c>
+      <c r="E148" t="s">
+        <v>37</v>
+      </c>
+      <c r="F148" t="s">
+        <v>8</v>
+      </c>
+      <c r="G148" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A149" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B149" t="s">
+        <v>338</v>
+      </c>
+      <c r="C149" t="s">
+        <v>339</v>
+      </c>
+      <c r="D149" t="s">
+        <v>15</v>
+      </c>
+      <c r="E149" t="s">
+        <v>37</v>
+      </c>
+      <c r="F149" t="s">
+        <v>8</v>
+      </c>
+      <c r="G149" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A150" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B150" t="s">
+        <v>340</v>
+      </c>
+      <c r="C150" t="s">
+        <v>341</v>
+      </c>
+      <c r="D150" t="s">
+        <v>16</v>
+      </c>
+      <c r="E150" t="s">
+        <v>37</v>
+      </c>
+      <c r="F150" t="s">
+        <v>8</v>
+      </c>
+      <c r="G150" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A151" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B151" t="s">
+        <v>342</v>
+      </c>
+      <c r="C151" t="s">
+        <v>343</v>
+      </c>
+      <c r="D151" t="s">
+        <v>28</v>
+      </c>
+      <c r="E151" t="s">
+        <v>37</v>
+      </c>
+      <c r="F151" t="s">
+        <v>8</v>
+      </c>
+      <c r="G151" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A152" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B152" t="s">
+        <v>344</v>
+      </c>
+      <c r="C152" t="s">
+        <v>345</v>
+      </c>
+      <c r="D152" t="s">
+        <v>14</v>
+      </c>
+      <c r="E152" t="s">
+        <v>37</v>
+      </c>
+      <c r="F152" t="s">
+        <v>8</v>
+      </c>
+      <c r="G152" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A153" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B153" t="s">
+        <v>346</v>
+      </c>
+      <c r="C153" t="s">
+        <v>347</v>
+      </c>
+      <c r="D153" t="s">
+        <v>31</v>
+      </c>
+      <c r="E153" t="s">
+        <v>39</v>
+      </c>
+      <c r="F153" t="s">
+        <v>8</v>
+      </c>
+      <c r="G153" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A154" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B154" t="s">
+        <v>348</v>
+      </c>
+      <c r="C154" t="s">
+        <v>349</v>
+      </c>
+      <c r="D154" t="s">
+        <v>16</v>
+      </c>
+      <c r="E154" t="s">
+        <v>37</v>
+      </c>
+      <c r="F154" t="s">
+        <v>8</v>
+      </c>
+      <c r="G154" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A155" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B155" t="s">
+        <v>350</v>
+      </c>
+      <c r="C155" t="s">
+        <v>351</v>
+      </c>
+      <c r="D155" t="s">
+        <v>11</v>
+      </c>
+      <c r="E155" t="s">
+        <v>37</v>
+      </c>
+      <c r="F155" t="s">
+        <v>8</v>
+      </c>
+      <c r="G155" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A156" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B156" t="s">
+        <v>352</v>
+      </c>
+      <c r="C156" t="s">
+        <v>353</v>
+      </c>
+      <c r="D156" t="s">
+        <v>14</v>
+      </c>
+      <c r="E156" t="s">
+        <v>37</v>
+      </c>
+      <c r="F156" t="s">
+        <v>8</v>
+      </c>
+      <c r="G156" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A157" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B157" t="s">
+        <v>354</v>
+      </c>
+      <c r="C157" t="s">
+        <v>355</v>
+      </c>
+      <c r="D157" t="s">
+        <v>31</v>
+      </c>
+      <c r="E157" t="s">
+        <v>39</v>
+      </c>
+      <c r="F157" t="s">
+        <v>8</v>
+      </c>
+      <c r="G157" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A158" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B158" t="s">
+        <v>356</v>
+      </c>
+      <c r="C158" t="s">
+        <v>357</v>
+      </c>
+      <c r="D158" t="s">
+        <v>11</v>
+      </c>
+      <c r="E158" t="s">
+        <v>37</v>
+      </c>
+      <c r="F158" t="s">
+        <v>8</v>
+      </c>
+      <c r="G158" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A159" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B159" t="s">
+        <v>358</v>
+      </c>
+      <c r="C159" t="s">
+        <v>359</v>
+      </c>
+      <c r="D159" t="s">
+        <v>22</v>
+      </c>
+      <c r="E159" t="s">
+        <v>39</v>
+      </c>
+      <c r="F159" t="s">
+        <v>8</v>
+      </c>
+      <c r="G159" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A160" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B160" t="s">
+        <v>360</v>
+      </c>
+      <c r="C160" t="s">
+        <v>361</v>
+      </c>
+      <c r="D160" t="s">
+        <v>24</v>
+      </c>
+      <c r="E160" t="s">
+        <v>39</v>
+      </c>
+      <c r="F160" t="s">
+        <v>7</v>
+      </c>
+      <c r="G160" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A161" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B161" t="s">
+        <v>362</v>
+      </c>
+      <c r="C161" t="s">
+        <v>363</v>
+      </c>
+      <c r="D161" t="s">
+        <v>6</v>
+      </c>
+      <c r="E161" t="s">
+        <v>37</v>
+      </c>
+      <c r="F161" t="s">
+        <v>8</v>
+      </c>
+      <c r="G161" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A162" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B162" t="s">
+        <v>364</v>
+      </c>
+      <c r="C162" t="s">
+        <v>365</v>
+      </c>
+      <c r="D162" t="s">
+        <v>14</v>
+      </c>
+      <c r="E162" t="s">
+        <v>37</v>
+      </c>
+      <c r="F162" t="s">
+        <v>8</v>
+      </c>
+      <c r="G162" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A163" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B163" t="s">
+        <v>366</v>
+      </c>
+      <c r="C163" t="s">
+        <v>367</v>
+      </c>
+      <c r="D163" t="s">
+        <v>40</v>
+      </c>
+      <c r="E163" t="s">
+        <v>39</v>
+      </c>
+      <c r="F163" t="s">
+        <v>7</v>
+      </c>
+      <c r="G163" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A164" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B164" t="s">
+        <v>368</v>
+      </c>
+      <c r="C164" t="s">
+        <v>369</v>
+      </c>
+      <c r="D164" t="s">
+        <v>25</v>
+      </c>
+      <c r="E164" t="s">
+        <v>39</v>
+      </c>
+      <c r="F164" t="s">
+        <v>7</v>
+      </c>
+      <c r="G164" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A165" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B165" t="s">
+        <v>370</v>
+      </c>
+      <c r="C165" t="s">
+        <v>371</v>
+      </c>
+      <c r="D165" t="s">
+        <v>14</v>
+      </c>
+      <c r="E165" t="s">
+        <v>37</v>
+      </c>
+      <c r="F165" t="s">
+        <v>8</v>
+      </c>
+      <c r="G165" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A166" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B166" t="s">
+        <v>372</v>
+      </c>
+      <c r="C166" t="s">
+        <v>373</v>
+      </c>
+      <c r="D166" t="s">
+        <v>19</v>
+      </c>
+      <c r="E166" t="s">
+        <v>37</v>
+      </c>
+      <c r="F166" t="s">
+        <v>8</v>
+      </c>
+      <c r="G166" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A167" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B167" t="s">
+        <v>374</v>
+      </c>
+      <c r="C167" t="s">
+        <v>375</v>
+      </c>
+      <c r="D167" t="s">
+        <v>11</v>
+      </c>
+      <c r="E167" t="s">
+        <v>37</v>
+      </c>
+      <c r="F167" t="s">
+        <v>8</v>
+      </c>
+      <c r="G167" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A168" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B168" t="s">
+        <v>376</v>
+      </c>
+      <c r="C168" t="s">
+        <v>377</v>
+      </c>
+      <c r="D168" t="s">
+        <v>24</v>
+      </c>
+      <c r="E168" t="s">
+        <v>39</v>
+      </c>
+      <c r="F168" t="s">
+        <v>8</v>
+      </c>
+      <c r="G168" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A169" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B169" t="s">
+        <v>378</v>
+      </c>
+      <c r="C169" t="s">
+        <v>379</v>
+      </c>
+      <c r="D169" t="s">
+        <v>40</v>
+      </c>
+      <c r="E169" t="s">
+        <v>39</v>
+      </c>
+      <c r="F169" t="s">
+        <v>7</v>
+      </c>
+      <c r="G169" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A170" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B170" t="s">
+        <v>380</v>
+      </c>
+      <c r="C170" t="s">
+        <v>381</v>
+      </c>
+      <c r="D170" t="s">
+        <v>15</v>
+      </c>
+      <c r="E170" t="s">
+        <v>37</v>
+      </c>
+      <c r="F170" t="s">
+        <v>8</v>
+      </c>
+      <c r="G170" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A171" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B171" t="s">
+        <v>382</v>
+      </c>
+      <c r="C171" t="s">
+        <v>383</v>
+      </c>
+      <c r="D171" t="s">
+        <v>15</v>
+      </c>
+      <c r="E171" t="s">
+        <v>37</v>
+      </c>
+      <c r="F171" t="s">
+        <v>8</v>
+      </c>
+      <c r="G171" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A172" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B172" t="s">
+        <v>384</v>
+      </c>
+      <c r="C172" t="s">
+        <v>385</v>
+      </c>
+      <c r="D172" t="s">
+        <v>22</v>
+      </c>
+      <c r="E172" t="s">
+        <v>39</v>
+      </c>
+      <c r="F172" t="s">
+        <v>8</v>
+      </c>
+      <c r="G172" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A173" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B173" t="s">
+        <v>386</v>
+      </c>
+      <c r="C173" t="s">
+        <v>387</v>
+      </c>
+      <c r="D173" t="s">
+        <v>11</v>
+      </c>
+      <c r="E173" t="s">
+        <v>37</v>
+      </c>
+      <c r="F173" t="s">
+        <v>8</v>
+      </c>
+      <c r="G173" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A174" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B174" t="s">
+        <v>388</v>
+      </c>
+      <c r="C174" t="s">
+        <v>389</v>
+      </c>
+      <c r="D174" t="s">
+        <v>12</v>
+      </c>
+      <c r="E174" t="s">
+        <v>37</v>
+      </c>
+      <c r="F174" t="s">
+        <v>8</v>
+      </c>
+      <c r="G174" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A175" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B175" t="s">
+        <v>390</v>
+      </c>
+      <c r="C175" t="s">
+        <v>391</v>
+      </c>
+      <c r="D175" t="s">
+        <v>12</v>
+      </c>
+      <c r="E175" t="s">
+        <v>37</v>
+      </c>
+      <c r="F175" t="s">
+        <v>392</v>
+      </c>
+      <c r="G175" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A176" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B176" t="s">
+        <v>393</v>
+      </c>
+      <c r="C176" t="s">
+        <v>394</v>
+      </c>
+      <c r="D176" t="s">
+        <v>23</v>
+      </c>
+      <c r="E176" t="s">
+        <v>37</v>
+      </c>
+      <c r="F176" t="s">
+        <v>8</v>
+      </c>
+      <c r="G176" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A177" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B177" t="s">
+        <v>395</v>
+      </c>
+      <c r="C177" t="s">
+        <v>396</v>
+      </c>
+      <c r="D177" t="s">
+        <v>14</v>
+      </c>
+      <c r="E177" t="s">
+        <v>37</v>
+      </c>
+      <c r="F177" t="s">
+        <v>8</v>
+      </c>
+      <c r="G177" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A178" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B178" t="s">
+        <v>397</v>
+      </c>
+      <c r="C178" t="s">
+        <v>398</v>
+      </c>
+      <c r="D178" t="s">
+        <v>28</v>
+      </c>
+      <c r="E178" t="s">
+        <v>37</v>
+      </c>
+      <c r="F178" t="s">
+        <v>8</v>
+      </c>
+      <c r="G178" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A179" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B179" t="s">
+        <v>399</v>
+      </c>
+      <c r="C179" t="s">
+        <v>400</v>
+      </c>
+      <c r="D179" t="s">
+        <v>19</v>
+      </c>
+      <c r="E179" t="s">
+        <v>37</v>
+      </c>
+      <c r="F179" t="s">
+        <v>392</v>
+      </c>
+      <c r="G179" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A180" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B180" t="s">
+        <v>401</v>
+      </c>
+      <c r="C180" t="s">
+        <v>402</v>
+      </c>
+      <c r="D180" t="s">
+        <v>15</v>
+      </c>
+      <c r="E180" t="s">
+        <v>37</v>
+      </c>
+      <c r="F180" t="s">
+        <v>8</v>
+      </c>
+      <c r="G180" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A181" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B181" t="s">
+        <v>403</v>
+      </c>
+      <c r="C181" t="s">
+        <v>404</v>
+      </c>
+      <c r="D181" t="s">
+        <v>15</v>
+      </c>
+      <c r="E181" t="s">
+        <v>37</v>
+      </c>
+      <c r="F181" t="s">
+        <v>8</v>
+      </c>
+      <c r="G181" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A182" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B182" t="s">
+        <v>405</v>
+      </c>
+      <c r="C182" t="s">
+        <v>406</v>
+      </c>
+      <c r="D182" t="s">
+        <v>24</v>
+      </c>
+      <c r="E182" t="s">
+        <v>39</v>
+      </c>
+      <c r="F182" t="s">
+        <v>7</v>
+      </c>
+      <c r="G182" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A183" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B183" t="s">
+        <v>407</v>
+      </c>
+      <c r="C183" t="s">
+        <v>408</v>
+      </c>
+      <c r="D183" t="s">
+        <v>6</v>
+      </c>
+      <c r="E183" t="s">
+        <v>37</v>
+      </c>
+      <c r="F183" t="s">
+        <v>8</v>
+      </c>
+      <c r="G183" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A184" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B184" t="s">
+        <v>409</v>
+      </c>
+      <c r="C184" t="s">
+        <v>410</v>
+      </c>
+      <c r="D184" t="s">
+        <v>25</v>
+      </c>
+      <c r="E184" t="s">
+        <v>39</v>
+      </c>
+      <c r="F184" t="s">
+        <v>7</v>
+      </c>
+      <c r="G184" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated balde and producao - base 08/04/2026
</commit_message>
<xml_diff>
--- a/first-atlas/producao_2026-04.xlsx
+++ b/first-atlas/producao_2026-04.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\augustoalmeida\Augusto\bots_comissionamento\bot_atlas\first-atlas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBFA352B-6409-4D08-A7F1-C669F9A2B4A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B8F060-660E-46A1-807D-14851B6658A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{F5572131-3C84-4D9C-B555-72DCC3B1940B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1951" uniqueCount="696">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2327" uniqueCount="824">
   <si>
     <t>DATA_BASE</t>
   </si>
@@ -2127,6 +2127,390 @@
   </si>
   <si>
     <t>Procuracao com poderes de abrir e movimentar conta corrente junto a instituicoes financeiras com mandato vigente e devidamente assinada&lt;br&gt;&lt;br&gt;Contrato Social atualizado e registrado no orgao competente</t>
+  </si>
+  <si>
+    <t>66119726000156</t>
+  </si>
+  <si>
+    <t>SAMUEL CHRISTO SOCIEDADE INDIVIDUAL DE ADVOCACIA</t>
+  </si>
+  <si>
+    <t>52201313000101</t>
+  </si>
+  <si>
+    <t>GIAN CARLOS</t>
+  </si>
+  <si>
+    <t>35329411000100</t>
+  </si>
+  <si>
+    <t>ATUAL SOLUCOES EMPRESARIAIS LTDA</t>
+  </si>
+  <si>
+    <t>41338993000193</t>
+  </si>
+  <si>
+    <t>AR INTERMEDIACOES E REPRESENTACOES LTDA</t>
+  </si>
+  <si>
+    <t>36411708000182</t>
+  </si>
+  <si>
+    <t>MARIA DA LUZ TRINDADE DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>62575959000102</t>
+  </si>
+  <si>
+    <t>TAYLOR KLEIN NUNES REPRESENTACOES</t>
+  </si>
+  <si>
+    <t>44961037000151</t>
+  </si>
+  <si>
+    <t>LEILA LIMA DO NASCIMENTO</t>
+  </si>
+  <si>
+    <t>39147133000120</t>
+  </si>
+  <si>
+    <t>JANETE DA APARECIDA DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>33157239000129</t>
+  </si>
+  <si>
+    <t>FABRICIO BERNARDINO DA SILVA</t>
+  </si>
+  <si>
+    <t>40410461000157</t>
+  </si>
+  <si>
+    <t>40.410.461 FRANCISCO DAS CHAGAS RODRIGUES</t>
+  </si>
+  <si>
+    <t>50813026000127</t>
+  </si>
+  <si>
+    <t>KAUAN MILHOMEM LIMA</t>
+  </si>
+  <si>
+    <t>65128920000135</t>
+  </si>
+  <si>
+    <t>M WEALTH E WELFARE ID LTDA</t>
+  </si>
+  <si>
+    <t>32018926000109</t>
+  </si>
+  <si>
+    <t>FLAVIO ALEXANDRE GIOIA CELESTE</t>
+  </si>
+  <si>
+    <t>44270036000160</t>
+  </si>
+  <si>
+    <t>PRISCILA MARIA LEALDINI</t>
+  </si>
+  <si>
+    <t>27642521000107</t>
+  </si>
+  <si>
+    <t>JOSE ROBERTO MEDEIROS BATISTA</t>
+  </si>
+  <si>
+    <t>54948362000138</t>
+  </si>
+  <si>
+    <t>FABIANA SINNES LTDA</t>
+  </si>
+  <si>
+    <t>60912849000163</t>
+  </si>
+  <si>
+    <t>V RODRIGUES DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>63645708000110</t>
+  </si>
+  <si>
+    <t>63.645.708 MOISES LAZARO DA ROCHA</t>
+  </si>
+  <si>
+    <t>61113487000103</t>
+  </si>
+  <si>
+    <t>F M DO VALE COMERCIO E SERVICOS</t>
+  </si>
+  <si>
+    <t>33721165000101</t>
+  </si>
+  <si>
+    <t>KATIA BARGIERI DE CARVALHO ROCHA GESTAO EMPRESARIAL</t>
+  </si>
+  <si>
+    <t>44068144000155</t>
+  </si>
+  <si>
+    <t>ALCIONE TORRES SENA ANDRADE</t>
+  </si>
+  <si>
+    <t>44127933000110</t>
+  </si>
+  <si>
+    <t>DAIANA LOPES TAVARES</t>
+  </si>
+  <si>
+    <t>18844706000103</t>
+  </si>
+  <si>
+    <t>CLAYTON NOEL DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>45796541000106</t>
+  </si>
+  <si>
+    <t>FRANCISCO JOSE FERNANDES ANDRE</t>
+  </si>
+  <si>
+    <t>34371846000150</t>
+  </si>
+  <si>
+    <t>IRINEU FRANCISCO DE LACERDA</t>
+  </si>
+  <si>
+    <t>35256355000120</t>
+  </si>
+  <si>
+    <t>ALDINETE RIBEIRO DA SILVA</t>
+  </si>
+  <si>
+    <t>19843526000161</t>
+  </si>
+  <si>
+    <t>PRECISA SOLUCOES EM MOVEIS PLANEJADOS LTDA</t>
+  </si>
+  <si>
+    <t>13721798000293</t>
+  </si>
+  <si>
+    <t>INSTITUTO SAO MIGUEL ARCANJO</t>
+  </si>
+  <si>
+    <t>61816926000144</t>
+  </si>
+  <si>
+    <t>J. OSMAR MARQUES DE SOUZA</t>
+  </si>
+  <si>
+    <t>47991920000182</t>
+  </si>
+  <si>
+    <t>DIONE DA SILVA LIMA</t>
+  </si>
+  <si>
+    <t>39591167000100</t>
+  </si>
+  <si>
+    <t>BRUNA NATALIA DO CARMO MAZZO PISSOLITO</t>
+  </si>
+  <si>
+    <t>55210134000129</t>
+  </si>
+  <si>
+    <t>ROSMERY SALCEDO APAZA</t>
+  </si>
+  <si>
+    <t>47505012000131</t>
+  </si>
+  <si>
+    <t>LUCIELE EVANGELISTA DA SILVA SANTOS</t>
+  </si>
+  <si>
+    <t>62376167000109</t>
+  </si>
+  <si>
+    <t>GLOBAL TRADE COMERCIO LTDA</t>
+  </si>
+  <si>
+    <t>RECADASTRO</t>
+  </si>
+  <si>
+    <t>49919722000133</t>
+  </si>
+  <si>
+    <t>49.919.722 DIEGO VIDAL DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>41568707000186</t>
+  </si>
+  <si>
+    <t>JUCIENE DOS SANTOS RODRIGUES</t>
+  </si>
+  <si>
+    <t>41010770000100</t>
+  </si>
+  <si>
+    <t>DOUGLAS SANTANA VAZ DE ALMEIDA</t>
+  </si>
+  <si>
+    <t>64860933000131</t>
+  </si>
+  <si>
+    <t>64.860.933 LUIZ GUSTAVO GONCALVES DOS SANTOS</t>
+  </si>
+  <si>
+    <t>35901411000132</t>
+  </si>
+  <si>
+    <t>ALBERTO RIAL DE POLY</t>
+  </si>
+  <si>
+    <t>53101078000169</t>
+  </si>
+  <si>
+    <t>E A PEREIRA DE SOUZA SERVICOS</t>
+  </si>
+  <si>
+    <t>73850240000159</t>
+  </si>
+  <si>
+    <t>P C A PONTES CONSTRUTORA LTDA</t>
+  </si>
+  <si>
+    <t>44456957000112</t>
+  </si>
+  <si>
+    <t>GGA ESFERAS DE VIDROS LTDA</t>
+  </si>
+  <si>
+    <t>63483572000199</t>
+  </si>
+  <si>
+    <t>F VALERIO LUCAS</t>
+  </si>
+  <si>
+    <t>56304711000295</t>
+  </si>
+  <si>
+    <t>M J LTDA</t>
+  </si>
+  <si>
+    <t>23348125000102</t>
+  </si>
+  <si>
+    <t>GABRIEL RODRIGUES DE MORAIS</t>
+  </si>
+  <si>
+    <t>43261885000195</t>
+  </si>
+  <si>
+    <t>43.261.885 MARILEIDE PEREIRA DAMACENA DA SILVA</t>
+  </si>
+  <si>
+    <t>65050309000131</t>
+  </si>
+  <si>
+    <t>JOSE CARLOS MAGALHAES PEREIRA JUNIOR</t>
+  </si>
+  <si>
+    <t>13439959000170</t>
+  </si>
+  <si>
+    <t>AUTO TOUR TRANSPORTES E TURISMO LTDA</t>
+  </si>
+  <si>
+    <t>57072165000196</t>
+  </si>
+  <si>
+    <t>57.072.165 ROBERIO SANTOS OLIVEIRA</t>
+  </si>
+  <si>
+    <t>47151283000136</t>
+  </si>
+  <si>
+    <t>ELEDIR ALDINO RONCEN CONSTRUCAO</t>
+  </si>
+  <si>
+    <t>20831856000116</t>
+  </si>
+  <si>
+    <t>GUINCHO CACHOEIRA LTDA</t>
+  </si>
+  <si>
+    <t>53863140000150</t>
+  </si>
+  <si>
+    <t>53.863.140 ANA PAULA GOMES</t>
+  </si>
+  <si>
+    <t>21721112000101</t>
+  </si>
+  <si>
+    <t>OMAR ROCHA REDA</t>
+  </si>
+  <si>
+    <t>36916501000160</t>
+  </si>
+  <si>
+    <t>36.916.501 MARCELO FONSECA FIDELIS</t>
+  </si>
+  <si>
+    <t>66084499000170</t>
+  </si>
+  <si>
+    <t>J F DA SILVA JOSE SYUVA COCHOES</t>
+  </si>
+  <si>
+    <t>27727193000133</t>
+  </si>
+  <si>
+    <t>27.727.193 JOSE CARNEIRO DE AGUIAR FILHO</t>
+  </si>
+  <si>
+    <t>35106276000133</t>
+  </si>
+  <si>
+    <t>KLEYVERTON DANTAS DE MEDEIROS</t>
+  </si>
+  <si>
+    <t>05017487000139</t>
+  </si>
+  <si>
+    <t>ASSOCIACAO CULTURAL E COMUNITARIA ZAGAIA</t>
+  </si>
+  <si>
+    <t>23656624000167</t>
+  </si>
+  <si>
+    <t>VERA LUCIA DE SOUSA SILVA</t>
+  </si>
+  <si>
+    <t>34185102000140</t>
+  </si>
+  <si>
+    <t>ESLEY ROSA PEREIRA</t>
+  </si>
+  <si>
+    <t>20598867000106</t>
+  </si>
+  <si>
+    <t>ANA CRISTINA SILVA DE SOUSA</t>
+  </si>
+  <si>
+    <t>54831244000145</t>
+  </si>
+  <si>
+    <t>MARIO SERGIO STROPARO</t>
+  </si>
+  <si>
+    <t>Para garantir a seguranca e a validade do processo. Pedimos gentilmente que envie uma nova foto apenas com voce, conforme as orientacoes.&lt;br&gt;&lt;br&gt;Procuracao da empresa , assinada via gov.br ou por meio de procuracao publica, em formato PDF. O documento deve conter, de forma expressa, os poderes para abrir e movimentar contas, alem de identificar corretamente o outorgante e o outorgado. Outorgante e a empresa (razao social) que concede os poderes</t>
+  </si>
+  <si>
+    <t>Procuracao da empresa , assinada via gov.br ou por meio de procuracao publica, em formato PDF. O documento deve conter, de forma expressa, os poderes para abrir e movimentar contas, alem de identificar corretamente o outorgante e o outorgado. Outorgante e a empresa (razao social) que concede os poderes</t>
+  </si>
+  <si>
+    <t>Ata de eleicao da diretoria atualizada e registrado no orgao competente&lt;br&gt;&lt;br&gt;Estatuto social atualizado e registrado no orgao competente</t>
   </si>
 </sst>
 </file>
@@ -2499,7 +2883,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39A45A88-3D17-4433-986A-11075963C36F}">
-  <dimension ref="A1:H324"/>
+  <dimension ref="A1:H386"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.28515625" style="1" bestFit="1" customWidth="1"/>
@@ -2741,10 +3125,10 @@
         <v>8</v>
       </c>
       <c r="G9" t="s">
-        <v>20</v>
+        <v>518</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>821</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -2975,10 +3359,10 @@
         <v>8</v>
       </c>
       <c r="G18" t="s">
-        <v>20</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
+        <v>518</v>
+      </c>
+      <c r="H18" t="s">
+        <v>822</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
@@ -5364,7 +5748,7 @@
         <v>7</v>
       </c>
       <c r="G110" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="H110">
         <v>0</v>
@@ -7513,7 +7897,7 @@
         <v>8</v>
       </c>
       <c r="G193" t="s">
-        <v>20</v>
+        <v>232</v>
       </c>
       <c r="H193">
         <v>0</v>
@@ -7718,7 +8102,7 @@
         <v>8</v>
       </c>
       <c r="G201" t="s">
-        <v>20</v>
+        <v>232</v>
       </c>
       <c r="H201">
         <v>0</v>
@@ -7978,7 +8362,7 @@
         <v>7</v>
       </c>
       <c r="G211" t="s">
-        <v>403</v>
+        <v>18</v>
       </c>
       <c r="H211">
         <v>0</v>
@@ -8394,7 +8778,7 @@
         <v>404</v>
       </c>
       <c r="G227" t="s">
-        <v>20</v>
+        <v>232</v>
       </c>
       <c r="H227">
         <v>0</v>
@@ -8420,7 +8804,7 @@
         <v>7</v>
       </c>
       <c r="G228" t="s">
-        <v>20</v>
+        <v>232</v>
       </c>
       <c r="H228">
         <v>0</v>
@@ -8628,7 +9012,7 @@
         <v>7</v>
       </c>
       <c r="G236" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H236">
         <v>0</v>
@@ -8838,6 +9222,9 @@
       <c r="G244" t="s">
         <v>18</v>
       </c>
+      <c r="H244">
+        <v>0</v>
+      </c>
     </row>
     <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245" s="1">
@@ -8861,6 +9248,9 @@
       <c r="G245" t="s">
         <v>18</v>
       </c>
+      <c r="H245">
+        <v>0</v>
+      </c>
     </row>
     <row r="246" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A246" s="1">
@@ -8884,6 +9274,9 @@
       <c r="G246" t="s">
         <v>18</v>
       </c>
+      <c r="H246">
+        <v>0</v>
+      </c>
     </row>
     <row r="247" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A247" s="1">
@@ -8905,7 +9298,10 @@
         <v>384</v>
       </c>
       <c r="G247" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="H247">
+        <v>0</v>
       </c>
     </row>
     <row r="248" spans="1:8" x14ac:dyDescent="0.25">
@@ -8930,6 +9326,9 @@
       <c r="G248" t="s">
         <v>21</v>
       </c>
+      <c r="H248">
+        <v>0</v>
+      </c>
     </row>
     <row r="249" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A249" s="1">
@@ -8953,6 +9352,9 @@
       <c r="G249" t="s">
         <v>18</v>
       </c>
+      <c r="H249">
+        <v>0</v>
+      </c>
     </row>
     <row r="250" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A250" s="1">
@@ -8999,6 +9401,9 @@
       <c r="G251" t="s">
         <v>18</v>
       </c>
+      <c r="H251">
+        <v>0</v>
+      </c>
     </row>
     <row r="252" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A252" s="1">
@@ -9022,6 +9427,9 @@
       <c r="G252" t="s">
         <v>18</v>
       </c>
+      <c r="H252">
+        <v>0</v>
+      </c>
     </row>
     <row r="253" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A253" s="1">
@@ -9045,6 +9453,9 @@
       <c r="G253" t="s">
         <v>18</v>
       </c>
+      <c r="H253">
+        <v>0</v>
+      </c>
     </row>
     <row r="254" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A254" s="1">
@@ -9068,6 +9479,9 @@
       <c r="G254" t="s">
         <v>18</v>
       </c>
+      <c r="H254">
+        <v>0</v>
+      </c>
     </row>
     <row r="255" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A255" s="1">
@@ -9091,6 +9505,9 @@
       <c r="G255" t="s">
         <v>18</v>
       </c>
+      <c r="H255">
+        <v>0</v>
+      </c>
     </row>
     <row r="256" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A256" s="1">
@@ -9114,8 +9531,11 @@
       <c r="G256" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H256">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A257" s="1">
         <v>46120</v>
       </c>
@@ -9137,8 +9557,11 @@
       <c r="G257" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H257">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A258" s="1">
         <v>46120</v>
       </c>
@@ -9160,8 +9583,11 @@
       <c r="G258" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H258">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A259" s="1">
         <v>46120</v>
       </c>
@@ -9183,8 +9609,11 @@
       <c r="G259" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H259">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A260" s="1">
         <v>46120</v>
       </c>
@@ -9206,8 +9635,11 @@
       <c r="G260" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H260">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A261" s="1">
         <v>46120</v>
       </c>
@@ -9229,8 +9661,11 @@
       <c r="G261" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H261">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A262" s="1">
         <v>46120</v>
       </c>
@@ -9250,10 +9685,10 @@
         <v>10</v>
       </c>
       <c r="G262" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A263" s="1">
         <v>46120</v>
       </c>
@@ -9275,8 +9710,11 @@
       <c r="G263" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H263">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A264" s="1">
         <v>46120</v>
       </c>
@@ -9296,10 +9734,13 @@
         <v>8</v>
       </c>
       <c r="G264" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+        <v>18</v>
+      </c>
+      <c r="H264">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A265" s="1">
         <v>46120</v>
       </c>
@@ -9321,8 +9762,11 @@
       <c r="G265" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H265">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A266" s="1">
         <v>46120</v>
       </c>
@@ -9344,8 +9788,11 @@
       <c r="G266" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H266">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A267" s="1">
         <v>46120</v>
       </c>
@@ -9367,8 +9814,11 @@
       <c r="G267" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H267">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A268" s="1">
         <v>46120</v>
       </c>
@@ -9390,8 +9840,11 @@
       <c r="G268" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H268">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A269" s="1">
         <v>46120</v>
       </c>
@@ -9413,8 +9866,11 @@
       <c r="G269" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H269">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A270" s="1">
         <v>46120</v>
       </c>
@@ -9434,10 +9890,13 @@
         <v>8</v>
       </c>
       <c r="G270" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+        <v>518</v>
+      </c>
+      <c r="H270" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A271" s="1">
         <v>46120</v>
       </c>
@@ -9459,8 +9918,11 @@
       <c r="G271" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H271">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A272" s="1">
         <v>46120</v>
       </c>
@@ -9482,8 +9944,11 @@
       <c r="G272" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H272">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A273" s="1">
         <v>46120</v>
       </c>
@@ -9505,8 +9970,11 @@
       <c r="G273" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H273">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A274" s="1">
         <v>46120</v>
       </c>
@@ -9528,8 +9996,11 @@
       <c r="G274" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H274">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A275" s="1">
         <v>46120</v>
       </c>
@@ -9551,8 +10022,11 @@
       <c r="G275" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H275">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A276" s="1">
         <v>46120</v>
       </c>
@@ -9574,8 +10048,11 @@
       <c r="G276" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H276">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A277" s="1">
         <v>46120</v>
       </c>
@@ -9597,8 +10074,11 @@
       <c r="G277" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H277">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A278" s="1">
         <v>46120</v>
       </c>
@@ -9620,8 +10100,11 @@
       <c r="G278" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H278">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A279" s="1">
         <v>46120</v>
       </c>
@@ -9643,8 +10126,11 @@
       <c r="G279" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H279">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A280" s="1">
         <v>46120</v>
       </c>
@@ -9666,8 +10152,11 @@
       <c r="G280" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H280">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A281" s="1">
         <v>46120</v>
       </c>
@@ -9689,8 +10178,11 @@
       <c r="G281" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H281">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A282" s="1">
         <v>46120</v>
       </c>
@@ -9712,8 +10204,11 @@
       <c r="G282" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H282">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A283" s="1">
         <v>46120</v>
       </c>
@@ -9735,8 +10230,11 @@
       <c r="G283" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H283">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A284" s="1">
         <v>46120</v>
       </c>
@@ -9758,8 +10256,11 @@
       <c r="G284" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H284">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A285" s="1">
         <v>46120</v>
       </c>
@@ -9781,8 +10282,11 @@
       <c r="G285" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H285">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A286" s="1">
         <v>46120</v>
       </c>
@@ -9804,8 +10308,11 @@
       <c r="G286" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H286">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A287" s="1">
         <v>46120</v>
       </c>
@@ -9827,8 +10334,11 @@
       <c r="G287" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H287">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A288" s="1">
         <v>46120</v>
       </c>
@@ -9850,8 +10360,11 @@
       <c r="G288" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H288">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A289" s="1">
         <v>46120</v>
       </c>
@@ -9873,8 +10386,11 @@
       <c r="G289" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H289">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A290" s="1">
         <v>46120</v>
       </c>
@@ -9896,8 +10412,11 @@
       <c r="G290" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H290">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A291" s="1">
         <v>46120</v>
       </c>
@@ -9919,8 +10438,11 @@
       <c r="G291" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H291">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A292" s="1">
         <v>46120</v>
       </c>
@@ -9942,8 +10464,11 @@
       <c r="G292" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H292">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A293" s="1">
         <v>46120</v>
       </c>
@@ -9963,10 +10488,13 @@
         <v>8</v>
       </c>
       <c r="G293" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+        <v>518</v>
+      </c>
+      <c r="H293" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A294" s="1">
         <v>46120</v>
       </c>
@@ -9988,8 +10516,11 @@
       <c r="G294" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H294">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A295" s="1">
         <v>46120</v>
       </c>
@@ -10011,8 +10542,11 @@
       <c r="G295" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H295">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A296" s="1">
         <v>46120</v>
       </c>
@@ -10034,8 +10568,11 @@
       <c r="G296" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H296">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A297" s="1">
         <v>46120</v>
       </c>
@@ -10057,8 +10594,11 @@
       <c r="G297" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H297">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A298" s="1">
         <v>46120</v>
       </c>
@@ -10080,8 +10620,11 @@
       <c r="G298" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H298">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A299" s="1">
         <v>46120</v>
       </c>
@@ -10103,8 +10646,11 @@
       <c r="G299" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H299">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A300" s="1">
         <v>46120</v>
       </c>
@@ -10126,8 +10672,11 @@
       <c r="G300" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H300">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A301" s="1">
         <v>46120</v>
       </c>
@@ -10149,8 +10698,11 @@
       <c r="G301" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H301">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302" s="1">
         <v>46120</v>
       </c>
@@ -10172,8 +10724,11 @@
       <c r="G302" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H302">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303" s="1">
         <v>46120</v>
       </c>
@@ -10195,8 +10750,11 @@
       <c r="G303" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H303">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A304" s="1">
         <v>46120</v>
       </c>
@@ -10218,8 +10776,11 @@
       <c r="G304" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H304">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A305" s="1">
         <v>46120</v>
       </c>
@@ -10241,8 +10802,11 @@
       <c r="G305" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H305">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A306" s="1">
         <v>46120</v>
       </c>
@@ -10264,8 +10828,11 @@
       <c r="G306" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H306">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307" s="1">
         <v>46120</v>
       </c>
@@ -10287,8 +10854,11 @@
       <c r="G307" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H307">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308" s="1">
         <v>46120</v>
       </c>
@@ -10310,8 +10880,11 @@
       <c r="G308" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H308">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309" s="1">
         <v>46120</v>
       </c>
@@ -10333,8 +10906,11 @@
       <c r="G309" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H309">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310" s="1">
         <v>46120</v>
       </c>
@@ -10356,8 +10932,11 @@
       <c r="G310" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H310">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A311" s="1">
         <v>46120</v>
       </c>
@@ -10379,8 +10958,11 @@
       <c r="G311" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H311">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A312" s="1">
         <v>46120</v>
       </c>
@@ -10402,8 +10984,11 @@
       <c r="G312" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H312">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A313" s="1">
         <v>46120</v>
       </c>
@@ -10425,8 +11010,11 @@
       <c r="G313" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H313">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A314" s="1">
         <v>46120</v>
       </c>
@@ -10448,8 +11036,11 @@
       <c r="G314" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="315" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H314">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A315" s="1">
         <v>46120</v>
       </c>
@@ -10471,8 +11062,11 @@
       <c r="G315" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="316" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H315">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A316" s="1">
         <v>46120</v>
       </c>
@@ -10494,8 +11088,11 @@
       <c r="G316" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H316">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A317" s="1">
         <v>46120</v>
       </c>
@@ -10517,8 +11114,11 @@
       <c r="G317" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="318" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H317">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A318" s="1">
         <v>46120</v>
       </c>
@@ -10540,8 +11140,11 @@
       <c r="G318" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="319" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H318">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A319" s="1">
         <v>46120</v>
       </c>
@@ -10561,10 +11164,13 @@
         <v>8</v>
       </c>
       <c r="G319" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="H319">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A320" s="1">
         <v>46120</v>
       </c>
@@ -10586,8 +11192,11 @@
       <c r="G320" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="321" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H320">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="321" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A321" s="1">
         <v>46120</v>
       </c>
@@ -10609,8 +11218,11 @@
       <c r="G321" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="322" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H321">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="322" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A322" s="1">
         <v>46120</v>
       </c>
@@ -10632,8 +11244,11 @@
       <c r="G322" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="323" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H322">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="323" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A323" s="1">
         <v>46120</v>
       </c>
@@ -10653,10 +11268,13 @@
         <v>8</v>
       </c>
       <c r="G323" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="324" spans="1:7" x14ac:dyDescent="0.25">
+        <v>518</v>
+      </c>
+      <c r="H323" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="324" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A324" s="1">
         <v>46120</v>
       </c>
@@ -10676,7 +11294,1445 @@
         <v>8</v>
       </c>
       <c r="G324" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="325" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A325" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B325" t="s">
+        <v>696</v>
+      </c>
+      <c r="C325" t="s">
+        <v>697</v>
+      </c>
+      <c r="D325" t="s">
+        <v>12</v>
+      </c>
+      <c r="E325" t="s">
+        <v>36</v>
+      </c>
+      <c r="F325" t="s">
+        <v>384</v>
+      </c>
+      <c r="G325" t="s">
+        <v>18</v>
+      </c>
+      <c r="H325">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="326" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A326" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B326" t="s">
+        <v>698</v>
+      </c>
+      <c r="C326" t="s">
+        <v>699</v>
+      </c>
+      <c r="D326" t="s">
+        <v>12</v>
+      </c>
+      <c r="E326" t="s">
+        <v>36</v>
+      </c>
+      <c r="F326" t="s">
+        <v>8</v>
+      </c>
+      <c r="G326" t="s">
+        <v>18</v>
+      </c>
+      <c r="H326">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="327" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A327" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B327" t="s">
+        <v>700</v>
+      </c>
+      <c r="C327" t="s">
+        <v>701</v>
+      </c>
+      <c r="D327" t="s">
+        <v>12</v>
+      </c>
+      <c r="E327" t="s">
+        <v>36</v>
+      </c>
+      <c r="F327" t="s">
+        <v>8</v>
+      </c>
+      <c r="G327" t="s">
+        <v>18</v>
+      </c>
+      <c r="H327">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="328" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A328" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B328" t="s">
+        <v>702</v>
+      </c>
+      <c r="C328" t="s">
+        <v>703</v>
+      </c>
+      <c r="D328" t="s">
+        <v>27</v>
+      </c>
+      <c r="E328" t="s">
+        <v>37</v>
+      </c>
+      <c r="F328" t="s">
+        <v>242</v>
+      </c>
+      <c r="G328" t="s">
+        <v>18</v>
+      </c>
+      <c r="H328">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="329" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A329" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B329" t="s">
+        <v>704</v>
+      </c>
+      <c r="C329" t="s">
+        <v>705</v>
+      </c>
+      <c r="D329" t="s">
+        <v>22</v>
+      </c>
+      <c r="E329" t="s">
+        <v>38</v>
+      </c>
+      <c r="F329" t="s">
+        <v>7</v>
+      </c>
+      <c r="G329" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="330" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A330" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B330" t="s">
+        <v>706</v>
+      </c>
+      <c r="C330" t="s">
+        <v>707</v>
+      </c>
+      <c r="D330" t="s">
+        <v>30</v>
+      </c>
+      <c r="E330" t="s">
+        <v>38</v>
+      </c>
+      <c r="F330" t="s">
+        <v>7</v>
+      </c>
+      <c r="G330" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="331" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A331" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B331" t="s">
+        <v>708</v>
+      </c>
+      <c r="C331" t="s">
+        <v>709</v>
+      </c>
+      <c r="D331" t="s">
+        <v>14</v>
+      </c>
+      <c r="E331" t="s">
+        <v>36</v>
+      </c>
+      <c r="F331" t="s">
+        <v>8</v>
+      </c>
+      <c r="G331" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="332" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A332" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B332" t="s">
+        <v>710</v>
+      </c>
+      <c r="C332" t="s">
+        <v>711</v>
+      </c>
+      <c r="D332" t="s">
+        <v>30</v>
+      </c>
+      <c r="E332" t="s">
+        <v>38</v>
+      </c>
+      <c r="F332" t="s">
+        <v>7</v>
+      </c>
+      <c r="G332" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A333" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B333" t="s">
+        <v>712</v>
+      </c>
+      <c r="C333" t="s">
+        <v>713</v>
+      </c>
+      <c r="D333" t="s">
+        <v>16</v>
+      </c>
+      <c r="E333" t="s">
+        <v>36</v>
+      </c>
+      <c r="F333" t="s">
+        <v>8</v>
+      </c>
+      <c r="G333" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="334" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A334" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B334" t="s">
+        <v>714</v>
+      </c>
+      <c r="C334" t="s">
+        <v>715</v>
+      </c>
+      <c r="D334" t="s">
+        <v>23</v>
+      </c>
+      <c r="E334" t="s">
+        <v>36</v>
+      </c>
+      <c r="F334" t="s">
+        <v>8</v>
+      </c>
+      <c r="G334" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="335" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A335" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B335" t="s">
+        <v>716</v>
+      </c>
+      <c r="C335" t="s">
+        <v>717</v>
+      </c>
+      <c r="D335" t="s">
+        <v>11</v>
+      </c>
+      <c r="E335" t="s">
+        <v>36</v>
+      </c>
+      <c r="F335" t="s">
+        <v>8</v>
+      </c>
+      <c r="G335" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="336" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A336" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B336" t="s">
+        <v>718</v>
+      </c>
+      <c r="C336" t="s">
+        <v>719</v>
+      </c>
+      <c r="D336" t="s">
+        <v>39</v>
+      </c>
+      <c r="E336" t="s">
+        <v>38</v>
+      </c>
+      <c r="F336" t="s">
+        <v>7</v>
+      </c>
+      <c r="G336" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="337" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A337" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B337" t="s">
+        <v>720</v>
+      </c>
+      <c r="C337" t="s">
+        <v>721</v>
+      </c>
+      <c r="D337" t="s">
+        <v>28</v>
+      </c>
+      <c r="E337" t="s">
+        <v>36</v>
+      </c>
+      <c r="F337" t="s">
+        <v>8</v>
+      </c>
+      <c r="G337" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="338" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A338" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B338" t="s">
+        <v>722</v>
+      </c>
+      <c r="C338" t="s">
+        <v>723</v>
+      </c>
+      <c r="D338" t="s">
+        <v>15</v>
+      </c>
+      <c r="E338" t="s">
+        <v>36</v>
+      </c>
+      <c r="F338" t="s">
+        <v>8</v>
+      </c>
+      <c r="G338" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="339" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A339" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B339" t="s">
+        <v>724</v>
+      </c>
+      <c r="C339" t="s">
+        <v>725</v>
+      </c>
+      <c r="D339" t="s">
+        <v>14</v>
+      </c>
+      <c r="E339" t="s">
+        <v>36</v>
+      </c>
+      <c r="F339" t="s">
+        <v>8</v>
+      </c>
+      <c r="G339" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="340" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A340" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B340" t="s">
+        <v>726</v>
+      </c>
+      <c r="C340" t="s">
+        <v>727</v>
+      </c>
+      <c r="D340" t="s">
+        <v>28</v>
+      </c>
+      <c r="E340" t="s">
+        <v>36</v>
+      </c>
+      <c r="F340" t="s">
+        <v>8</v>
+      </c>
+      <c r="G340" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="341" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A341" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B341" t="s">
+        <v>728</v>
+      </c>
+      <c r="C341" t="s">
+        <v>729</v>
+      </c>
+      <c r="D341" t="s">
+        <v>11</v>
+      </c>
+      <c r="E341" t="s">
+        <v>36</v>
+      </c>
+      <c r="F341" t="s">
+        <v>8</v>
+      </c>
+      <c r="G341" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="342" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A342" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B342" t="s">
+        <v>730</v>
+      </c>
+      <c r="C342" t="s">
+        <v>731</v>
+      </c>
+      <c r="D342" t="s">
+        <v>23</v>
+      </c>
+      <c r="E342" t="s">
+        <v>36</v>
+      </c>
+      <c r="F342" t="s">
+        <v>8</v>
+      </c>
+      <c r="G342" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="343" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A343" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B343" t="s">
+        <v>732</v>
+      </c>
+      <c r="C343" t="s">
+        <v>733</v>
+      </c>
+      <c r="D343" t="s">
+        <v>9</v>
+      </c>
+      <c r="E343" t="s">
+        <v>38</v>
+      </c>
+      <c r="F343" t="s">
+        <v>7</v>
+      </c>
+      <c r="G343" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="344" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A344" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B344" t="s">
+        <v>734</v>
+      </c>
+      <c r="C344" t="s">
+        <v>735</v>
+      </c>
+      <c r="D344" t="s">
+        <v>19</v>
+      </c>
+      <c r="E344" t="s">
+        <v>36</v>
+      </c>
+      <c r="F344" t="s">
+        <v>384</v>
+      </c>
+      <c r="G344" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="345" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A345" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B345" t="s">
+        <v>736</v>
+      </c>
+      <c r="C345" t="s">
+        <v>737</v>
+      </c>
+      <c r="D345" t="s">
+        <v>15</v>
+      </c>
+      <c r="E345" t="s">
+        <v>36</v>
+      </c>
+      <c r="F345" t="s">
+        <v>8</v>
+      </c>
+      <c r="G345" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="346" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A346" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B346" t="s">
+        <v>738</v>
+      </c>
+      <c r="C346" t="s">
+        <v>739</v>
+      </c>
+      <c r="D346" t="s">
+        <v>28</v>
+      </c>
+      <c r="E346" t="s">
+        <v>36</v>
+      </c>
+      <c r="F346" t="s">
+        <v>8</v>
+      </c>
+      <c r="G346" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="347" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A347" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B347" t="s">
+        <v>740</v>
+      </c>
+      <c r="C347" t="s">
+        <v>741</v>
+      </c>
+      <c r="D347" t="s">
+        <v>24</v>
+      </c>
+      <c r="E347" t="s">
+        <v>38</v>
+      </c>
+      <c r="F347" t="s">
+        <v>7</v>
+      </c>
+      <c r="G347" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="348" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A348" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B348" t="s">
+        <v>742</v>
+      </c>
+      <c r="C348" t="s">
+        <v>743</v>
+      </c>
+      <c r="D348" t="s">
+        <v>11</v>
+      </c>
+      <c r="E348" t="s">
+        <v>36</v>
+      </c>
+      <c r="F348" t="s">
+        <v>8</v>
+      </c>
+      <c r="G348" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="349" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A349" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B349" t="s">
+        <v>744</v>
+      </c>
+      <c r="C349" t="s">
+        <v>745</v>
+      </c>
+      <c r="D349" t="s">
+        <v>9</v>
+      </c>
+      <c r="E349" t="s">
+        <v>38</v>
+      </c>
+      <c r="F349" t="s">
+        <v>7</v>
+      </c>
+      <c r="G349" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="350" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A350" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B350" t="s">
+        <v>746</v>
+      </c>
+      <c r="C350" t="s">
+        <v>747</v>
+      </c>
+      <c r="D350" t="s">
+        <v>12</v>
+      </c>
+      <c r="E350" t="s">
+        <v>36</v>
+      </c>
+      <c r="F350" t="s">
+        <v>7</v>
+      </c>
+      <c r="G350" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="351" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A351" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B351" t="s">
+        <v>748</v>
+      </c>
+      <c r="C351" t="s">
+        <v>749</v>
+      </c>
+      <c r="D351" t="s">
+        <v>19</v>
+      </c>
+      <c r="E351" t="s">
+        <v>36</v>
+      </c>
+      <c r="F351" t="s">
+        <v>384</v>
+      </c>
+      <c r="G351" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="352" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A352" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B352" t="s">
+        <v>750</v>
+      </c>
+      <c r="C352" t="s">
+        <v>751</v>
+      </c>
+      <c r="D352" t="s">
+        <v>40</v>
+      </c>
+      <c r="E352" t="s">
+        <v>38</v>
+      </c>
+      <c r="F352" t="s">
+        <v>10</v>
+      </c>
+      <c r="G352" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="353" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A353" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B353" t="s">
+        <v>752</v>
+      </c>
+      <c r="C353" t="s">
+        <v>753</v>
+      </c>
+      <c r="D353" t="s">
+        <v>39</v>
+      </c>
+      <c r="E353" t="s">
+        <v>38</v>
+      </c>
+      <c r="F353" t="s">
+        <v>7</v>
+      </c>
+      <c r="G353" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="354" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A354" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B354" t="s">
+        <v>754</v>
+      </c>
+      <c r="C354" t="s">
+        <v>755</v>
+      </c>
+      <c r="D354" t="s">
+        <v>6</v>
+      </c>
+      <c r="E354" t="s">
+        <v>36</v>
+      </c>
+      <c r="F354" t="s">
+        <v>7</v>
+      </c>
+      <c r="G354" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="355" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A355" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B355" t="s">
+        <v>756</v>
+      </c>
+      <c r="C355" t="s">
+        <v>757</v>
+      </c>
+      <c r="D355" t="s">
+        <v>28</v>
+      </c>
+      <c r="E355" t="s">
+        <v>36</v>
+      </c>
+      <c r="F355" t="s">
+        <v>8</v>
+      </c>
+      <c r="G355" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="356" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A356" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B356" t="s">
+        <v>758</v>
+      </c>
+      <c r="C356" t="s">
+        <v>759</v>
+      </c>
+      <c r="D356" t="s">
+        <v>30</v>
+      </c>
+      <c r="E356" t="s">
+        <v>38</v>
+      </c>
+      <c r="F356" t="s">
+        <v>7</v>
+      </c>
+      <c r="G356" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="357" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A357" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B357" t="s">
+        <v>760</v>
+      </c>
+      <c r="C357" t="s">
+        <v>761</v>
+      </c>
+      <c r="D357" t="s">
+        <v>30</v>
+      </c>
+      <c r="E357" t="s">
+        <v>38</v>
+      </c>
+      <c r="F357" t="s">
+        <v>7</v>
+      </c>
+      <c r="G357" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="358" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A358" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B358" t="s">
+        <v>762</v>
+      </c>
+      <c r="C358" t="s">
+        <v>763</v>
+      </c>
+      <c r="D358" t="s">
+        <v>39</v>
+      </c>
+      <c r="E358" t="s">
+        <v>38</v>
+      </c>
+      <c r="F358" t="s">
+        <v>764</v>
+      </c>
+      <c r="G358" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="359" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A359" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B359" t="s">
+        <v>765</v>
+      </c>
+      <c r="C359" t="s">
+        <v>766</v>
+      </c>
+      <c r="D359" t="s">
+        <v>12</v>
+      </c>
+      <c r="E359" t="s">
+        <v>36</v>
+      </c>
+      <c r="F359" t="s">
+        <v>8</v>
+      </c>
+      <c r="G359" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="360" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A360" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B360" t="s">
+        <v>767</v>
+      </c>
+      <c r="C360" t="s">
+        <v>768</v>
+      </c>
+      <c r="D360" t="s">
+        <v>16</v>
+      </c>
+      <c r="E360" t="s">
+        <v>36</v>
+      </c>
+      <c r="F360" t="s">
+        <v>7</v>
+      </c>
+      <c r="G360" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="361" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A361" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B361" t="s">
+        <v>769</v>
+      </c>
+      <c r="C361" t="s">
+        <v>770</v>
+      </c>
+      <c r="D361" t="s">
+        <v>15</v>
+      </c>
+      <c r="E361" t="s">
+        <v>36</v>
+      </c>
+      <c r="F361" t="s">
+        <v>764</v>
+      </c>
+      <c r="G361" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="362" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A362" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B362" t="s">
+        <v>771</v>
+      </c>
+      <c r="C362" t="s">
+        <v>772</v>
+      </c>
+      <c r="D362" t="s">
+        <v>22</v>
+      </c>
+      <c r="E362" t="s">
+        <v>38</v>
+      </c>
+      <c r="F362" t="s">
+        <v>8</v>
+      </c>
+      <c r="G362" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="363" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A363" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B363" t="s">
+        <v>773</v>
+      </c>
+      <c r="C363" t="s">
+        <v>774</v>
+      </c>
+      <c r="D363" t="s">
+        <v>14</v>
+      </c>
+      <c r="E363" t="s">
+        <v>36</v>
+      </c>
+      <c r="F363" t="s">
+        <v>8</v>
+      </c>
+      <c r="G363" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="364" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A364" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B364" t="s">
+        <v>775</v>
+      </c>
+      <c r="C364" t="s">
+        <v>776</v>
+      </c>
+      <c r="D364" t="s">
+        <v>15</v>
+      </c>
+      <c r="E364" t="s">
+        <v>36</v>
+      </c>
+      <c r="F364" t="s">
+        <v>8</v>
+      </c>
+      <c r="G364" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="365" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A365" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B365" t="s">
+        <v>777</v>
+      </c>
+      <c r="C365" t="s">
+        <v>778</v>
+      </c>
+      <c r="D365" t="s">
+        <v>24</v>
+      </c>
+      <c r="E365" t="s">
+        <v>38</v>
+      </c>
+      <c r="F365" t="s">
+        <v>764</v>
+      </c>
+      <c r="G365" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="366" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A366" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B366" t="s">
+        <v>779</v>
+      </c>
+      <c r="C366" t="s">
+        <v>780</v>
+      </c>
+      <c r="D366" t="s">
+        <v>22</v>
+      </c>
+      <c r="E366" t="s">
+        <v>38</v>
+      </c>
+      <c r="F366" t="s">
+        <v>8</v>
+      </c>
+      <c r="G366" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="367" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A367" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B367" t="s">
+        <v>781</v>
+      </c>
+      <c r="C367" t="s">
+        <v>782</v>
+      </c>
+      <c r="D367" t="s">
+        <v>14</v>
+      </c>
+      <c r="E367" t="s">
+        <v>36</v>
+      </c>
+      <c r="F367" t="s">
+        <v>8</v>
+      </c>
+      <c r="G367" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="368" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A368" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B368" t="s">
+        <v>783</v>
+      </c>
+      <c r="C368" t="s">
+        <v>784</v>
+      </c>
+      <c r="D368" t="s">
+        <v>23</v>
+      </c>
+      <c r="E368" t="s">
+        <v>36</v>
+      </c>
+      <c r="F368" t="s">
+        <v>8</v>
+      </c>
+      <c r="G368" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="369" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A369" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B369" t="s">
+        <v>785</v>
+      </c>
+      <c r="C369" t="s">
+        <v>786</v>
+      </c>
+      <c r="D369" t="s">
+        <v>11</v>
+      </c>
+      <c r="E369" t="s">
+        <v>36</v>
+      </c>
+      <c r="F369" t="s">
+        <v>8</v>
+      </c>
+      <c r="G369" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="370" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A370" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B370" t="s">
+        <v>787</v>
+      </c>
+      <c r="C370" t="s">
+        <v>788</v>
+      </c>
+      <c r="D370" t="s">
+        <v>22</v>
+      </c>
+      <c r="E370" t="s">
+        <v>38</v>
+      </c>
+      <c r="F370" t="s">
+        <v>8</v>
+      </c>
+      <c r="G370" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="371" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A371" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B371" t="s">
+        <v>789</v>
+      </c>
+      <c r="C371" t="s">
+        <v>790</v>
+      </c>
+      <c r="D371" t="s">
+        <v>11</v>
+      </c>
+      <c r="E371" t="s">
+        <v>36</v>
+      </c>
+      <c r="F371" t="s">
+        <v>8</v>
+      </c>
+      <c r="G371" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="372" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A372" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B372" t="s">
+        <v>791</v>
+      </c>
+      <c r="C372" t="s">
+        <v>792</v>
+      </c>
+      <c r="D372" t="s">
+        <v>25</v>
+      </c>
+      <c r="E372" t="s">
+        <v>38</v>
+      </c>
+      <c r="F372" t="s">
+        <v>10</v>
+      </c>
+      <c r="G372" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="373" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A373" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B373" t="s">
+        <v>793</v>
+      </c>
+      <c r="C373" t="s">
+        <v>794</v>
+      </c>
+      <c r="D373" t="s">
+        <v>14</v>
+      </c>
+      <c r="E373" t="s">
+        <v>36</v>
+      </c>
+      <c r="F373" t="s">
+        <v>8</v>
+      </c>
+      <c r="G373" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="374" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A374" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B374" t="s">
+        <v>795</v>
+      </c>
+      <c r="C374" t="s">
+        <v>796</v>
+      </c>
+      <c r="D374" t="s">
+        <v>24</v>
+      </c>
+      <c r="E374" t="s">
+        <v>38</v>
+      </c>
+      <c r="F374" t="s">
+        <v>8</v>
+      </c>
+      <c r="G374" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="375" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A375" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B375" t="s">
+        <v>797</v>
+      </c>
+      <c r="C375" t="s">
+        <v>798</v>
+      </c>
+      <c r="D375" t="s">
+        <v>28</v>
+      </c>
+      <c r="E375" t="s">
+        <v>36</v>
+      </c>
+      <c r="F375" t="s">
+        <v>8</v>
+      </c>
+      <c r="G375" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="376" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A376" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B376" t="s">
+        <v>799</v>
+      </c>
+      <c r="C376" t="s">
+        <v>800</v>
+      </c>
+      <c r="D376" t="s">
+        <v>16</v>
+      </c>
+      <c r="E376" t="s">
+        <v>36</v>
+      </c>
+      <c r="F376" t="s">
+        <v>8</v>
+      </c>
+      <c r="G376" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="377" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A377" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B377" t="s">
+        <v>801</v>
+      </c>
+      <c r="C377" t="s">
+        <v>802</v>
+      </c>
+      <c r="D377" t="s">
+        <v>16</v>
+      </c>
+      <c r="E377" t="s">
+        <v>36</v>
+      </c>
+      <c r="F377" t="s">
+        <v>8</v>
+      </c>
+      <c r="G377" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="378" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A378" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B378" t="s">
+        <v>803</v>
+      </c>
+      <c r="C378" t="s">
+        <v>804</v>
+      </c>
+      <c r="D378" t="s">
+        <v>16</v>
+      </c>
+      <c r="E378" t="s">
+        <v>36</v>
+      </c>
+      <c r="F378" t="s">
+        <v>8</v>
+      </c>
+      <c r="G378" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="379" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A379" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B379" t="s">
+        <v>805</v>
+      </c>
+      <c r="C379" t="s">
+        <v>806</v>
+      </c>
+      <c r="D379" t="s">
+        <v>23</v>
+      </c>
+      <c r="E379" t="s">
+        <v>36</v>
+      </c>
+      <c r="F379" t="s">
+        <v>8</v>
+      </c>
+      <c r="G379" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="380" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A380" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B380" t="s">
+        <v>807</v>
+      </c>
+      <c r="C380" t="s">
+        <v>808</v>
+      </c>
+      <c r="D380" t="s">
+        <v>30</v>
+      </c>
+      <c r="E380" t="s">
+        <v>38</v>
+      </c>
+      <c r="F380" t="s">
+        <v>8</v>
+      </c>
+      <c r="G380" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="381" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A381" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B381" t="s">
+        <v>809</v>
+      </c>
+      <c r="C381" t="s">
+        <v>810</v>
+      </c>
+      <c r="D381" t="s">
+        <v>11</v>
+      </c>
+      <c r="E381" t="s">
+        <v>36</v>
+      </c>
+      <c r="F381" t="s">
+        <v>8</v>
+      </c>
+      <c r="G381" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="382" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A382" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B382" t="s">
+        <v>811</v>
+      </c>
+      <c r="C382" t="s">
+        <v>812</v>
+      </c>
+      <c r="D382" t="s">
+        <v>22</v>
+      </c>
+      <c r="E382" t="s">
+        <v>38</v>
+      </c>
+      <c r="F382" t="s">
+        <v>8</v>
+      </c>
+      <c r="G382" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="383" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A383" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B383" t="s">
+        <v>813</v>
+      </c>
+      <c r="C383" t="s">
+        <v>814</v>
+      </c>
+      <c r="D383" t="s">
+        <v>15</v>
+      </c>
+      <c r="E383" t="s">
+        <v>36</v>
+      </c>
+      <c r="F383" t="s">
+        <v>8</v>
+      </c>
+      <c r="G383" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="384" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A384" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B384" t="s">
+        <v>815</v>
+      </c>
+      <c r="C384" t="s">
+        <v>816</v>
+      </c>
+      <c r="D384" t="s">
+        <v>261</v>
+      </c>
+      <c r="E384" t="s">
+        <v>36</v>
+      </c>
+      <c r="F384" t="s">
+        <v>8</v>
+      </c>
+      <c r="G384" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="385" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A385" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B385" t="s">
+        <v>817</v>
+      </c>
+      <c r="C385" t="s">
+        <v>818</v>
+      </c>
+      <c r="D385" t="s">
+        <v>28</v>
+      </c>
+      <c r="E385" t="s">
+        <v>36</v>
+      </c>
+      <c r="F385" t="s">
+        <v>8</v>
+      </c>
+      <c r="G385" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="386" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A386" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B386" t="s">
+        <v>819</v>
+      </c>
+      <c r="C386" t="s">
+        <v>820</v>
+      </c>
+      <c r="D386" t="s">
+        <v>11</v>
+      </c>
+      <c r="E386" t="s">
+        <v>36</v>
+      </c>
+      <c r="F386" t="s">
+        <v>8</v>
+      </c>
+      <c r="G386" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>